<commit_message>
Compare 23 September meter readings with today's photos for Fundo Zapallar.
Uses the validation-report photos as the baseline and sets the register difference against the same complete-hour WES window.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -1,31 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lecturas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Horario hoy" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Historico mensual" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Cierre de indice" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Hallazgos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relojeria" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lecturas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horario hoy" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historico mensual" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cierre de indice" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hallazgos" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$5:$C$22</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Resumen'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lecturas'!$A$4:$C$22</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Lecturas'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Horario hoy'!$A$4:$E$18</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Horario hoy'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Historico mensual'!$A$4:$G$21</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Historico mensual'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Cierre de indice'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Hallazgos'!$A$4:$D$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Hallazgos'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relojeria'!$A$4:$J$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Relojeria'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resumen'!$A$5:$C$22</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Resumen'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lecturas'!$A$4:$C$22</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Lecturas'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Horario hoy'!$A$4:$E$19</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Horario hoy'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historico mensual'!$A$4:$G$21</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Historico mensual'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Cierre de indice'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Hallazgos'!$A$4:$D$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Hallazgos'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36,7 +39,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,8 +89,14 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="18"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -106,12 +115,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -134,8 +143,13 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -157,11 +171,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -213,9 +271,9 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -239,6 +297,18 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -249,18 +319,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -301,22 +359,50 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -394,14 +480,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -425,7 +510,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -449,7 +534,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -488,8 +573,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -516,7 +601,62 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9334500" cy="5905500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9334500" cy="5905500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -531,9 +671,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -828,6 +968,236 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E79"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>Diferencia de relojería  ·  23-09-2026 contra las fotos de hoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>Fotos de inicio rescatadas del informe de validación (23-09-2026). La app suma las horas completas del CSV, con la marca TIME en hora Chile, y deja fuera la hora de la foto final. Es la misma regla del cierre 23–28/09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="61" t="inlineStr">
+        <is>
+          <t>Punto</t>
+        </is>
+      </c>
+      <c r="B4" s="61" t="inlineStr">
+        <is>
+          <t>Lectura 23-09 (m³)</t>
+        </is>
+      </c>
+      <c r="C4" s="61" t="inlineStr">
+        <is>
+          <t>Hora 23-09</t>
+        </is>
+      </c>
+      <c r="D4" s="61" t="inlineStr">
+        <is>
+          <t>Lectura hoy (m³)</t>
+        </is>
+      </c>
+      <c r="E4" s="61" t="inlineStr">
+        <is>
+          <t>Hora hoy</t>
+        </is>
+      </c>
+      <c r="F4" s="61" t="inlineStr">
+        <is>
+          <t>Δ relojería (m³)</t>
+        </is>
+      </c>
+      <c r="G4" s="61" t="inlineStr">
+        <is>
+          <t>App WES (m³)</t>
+        </is>
+      </c>
+      <c r="H4" s="61" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="I4" s="61" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="J4" s="61" t="inlineStr">
+        <is>
+          <t>Lectura</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="55" t="inlineStr">
+        <is>
+          <t>Etapa N°5  000027-03</t>
+        </is>
+      </c>
+      <c r="B5" s="62" t="n">
+        <v>5177</v>
+      </c>
+      <c r="C5" s="63" t="inlineStr">
+        <is>
+          <t>23-09-2026 16:54</t>
+        </is>
+      </c>
+      <c r="D5" s="62" t="n">
+        <v>5316.8</v>
+      </c>
+      <c r="E5" s="63" t="inlineStr">
+        <is>
+          <t>02-10-2026 08:44</t>
+        </is>
+      </c>
+      <c r="F5" s="62" t="n">
+        <v>139.8000000000002</v>
+      </c>
+      <c r="G5" s="62" t="n">
+        <v>195.6</v>
+      </c>
+      <c r="H5" s="64" t="n">
+        <v>207</v>
+      </c>
+      <c r="I5" s="35" t="n">
+        <v>0.2852760736196309</v>
+      </c>
+      <c r="J5" s="33" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="53" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL  000027-01</t>
+        </is>
+      </c>
+      <c r="B6" s="65" t="n">
+        <v>384148.9</v>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>23-09-2026 17:05</t>
+        </is>
+      </c>
+      <c r="D6" s="65" t="n">
+        <v>385430.8</v>
+      </c>
+      <c r="E6" s="54" t="inlineStr">
+        <is>
+          <t>02-10-2026 13:22</t>
+        </is>
+      </c>
+      <c r="F6" s="65" t="n">
+        <v>1281.899999999965</v>
+      </c>
+      <c r="G6" s="65" t="n">
+        <v>1309.56</v>
+      </c>
+      <c r="H6" s="66" t="n">
+        <v>212</v>
+      </c>
+      <c r="I6" s="31" t="n">
+        <v>0.0211215980940429</v>
+      </c>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>Estanque Inferior en la misma ventana de la Matriz: 1.133,4 m³ (87 % de la app, 212 horas). En el cierre 23–28/09 ese porcentaje era 87 %.</t>
+        </is>
+      </c>
+      <c r="B7" s="68" t="n"/>
+      <c r="C7" s="68" t="n"/>
+      <c r="D7" s="68" t="n"/>
+      <c r="E7" s="68" t="n"/>
+      <c r="F7" s="68" t="n"/>
+      <c r="G7" s="68" t="n"/>
+      <c r="H7" s="68" t="n"/>
+      <c r="I7" s="68" t="n"/>
+      <c r="J7" s="68" t="n"/>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Etapa N°5. El 23–28/09 este Sensus cerró en 0,8 % (48 m³ de relojería contra 47,6 m³ de app). Del 23-09 al 02-10 la app queda 55,8 m³ por encima de la relojería. El desvío es posterior al 28-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL. Error 2,1 % (app por encima del Itron), del mismo sentido y menor que el 3,7 % del 23–28/09. La telemetría de la Matriz sigue cortada desde las 13:14, por eso la hora 13 de hoy no entra en la suma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Las fotos de la izquierda salen del informe de validación del 23-09. Las de la derecha son las de hoy. La diferencia está puesta sobre esas mismas imágenes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1"/>
+  </sheetData>
+  <autoFilter ref="A4:J6"/>
+  <mergeCells count="6">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="A11:J11"/>
+  </mergeCells>
+  <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LWES · Fundo Zapallar · relojería 23-09 a 02-10&amp;RPágina &amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001F4788"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -854,7 +1224,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fotos del 02-10-2026  ·  Consulta WES 02-10-2026 13:49 hora Chile  ·  Empresa 000027</t>
+          <t>Fotos del 02-10-2026  ·  Consulta WES 02-10-2026 14:25 hora Chile  ·  Empresa 000027</t>
         </is>
       </c>
     </row>
@@ -1025,10 +1395,10 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>15316.8</v>
+        <v>5316.8</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>365430.85</v>
+        <v>385430.8</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
@@ -1039,12 +1409,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>015316 m³; décima girando de 8 a 9; aguja entre 7 y 8</t>
+          <t>005316 m³; décima girando de 8 a 9. Mismo odómetro que el 5.177 del 23-09</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>365430 m³; rodillos rojos 8 y 5; aguja ×0,001 entre 3 y 4</t>
+          <t>385430 m³; rodillo rojo 8. Mismo medidor que el 384.148,9 del 23-09</t>
         </is>
       </c>
     </row>
@@ -1073,12 +1443,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>021026 13:49</t>
+          <t>021026 14:25</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>021026 13:14</t>
+          <t>021026 14:14</t>
         </is>
       </c>
     </row>
@@ -1089,10 +1459,10 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>4.21</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -1105,7 +1475,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
@@ -1115,10 +1485,10 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.3</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>133.47</v>
+        <v>139.6</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
@@ -1142,12 +1512,12 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Medidor y pulso coinciden con el punto. Sigue transmitiendo.</t>
+          <t>Odómetro 005316,8. Contra el 5.177 del 23-09 la relojería avanza 139,8 m³ y la app suma 195,6 m³.</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Medidor corresponde a la matriz. La telemetría está detenida desde las 13:14.</t>
+          <t>Odómetro 385.430,8. Contra el 384.148,9 del 23-09 la relojería avanza 1.281,9 m³ y la app suma 1.309,6 m³.</t>
         </is>
       </c>
     </row>
@@ -1161,14 +1531,14 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Etapa N°5: seis rodillos en 015316 y el rodillo rojo de las décimas entre 8 y 9. La aguja del dial auxiliar queda entre 7 y 8. Se registra 15.316,8 m³.</t>
+          <t>Etapa N°5: el mismo Sensus del informe del 23-09 (odómetro 005177). Hoy los rodillos marcan 005316 y la décima está entre 8 y 9. Se registra 5.316,8 m³.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Matriz ESVAL: rodillos negros 365430, dos rodillos rojos en 8 y 5, aguja del dial ×0,001 entre 3 y 4. Se registra 365.430,85 m³.</t>
+          <t>Matriz ESVAL: el mismo Itron del informe del 23-09 (384.148,9 m³). Hoy los rodillos negros marcan 385430 y el rojo 8. Se registra 385.430,8 m³.</t>
         </is>
       </c>
     </row>
@@ -1248,14 +1618,14 @@
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>021026 13:14</t>
+          <t>021026 14:14</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>4.21</v>
+        <v>0.11</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
@@ -1281,11 +1651,11 @@
       </c>
       <c r="D33" s="14" t="inlineStr">
         <is>
-          <t>021026 13:47</t>
+          <t>021026 14:25</t>
         </is>
       </c>
       <c r="E33" s="16" t="n">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="F33" s="17" t="n">
         <v>0</v>
@@ -1314,11 +1684,11 @@
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>021026 13:49</t>
+          <t>021026 14:25</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>0</v>
@@ -1347,14 +1717,14 @@
       </c>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>021026 13:44</t>
+          <t>021026 14:25</t>
         </is>
       </c>
       <c r="E35" s="16" t="n">
-        <v>3.04</v>
+        <v>1.53</v>
       </c>
       <c r="F35" s="17" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="G35" s="18" t="inlineStr">
         <is>
@@ -1363,17 +1733,17 @@
       </c>
     </row>
     <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>La Matriz ESVAL quedó en la trama de las 13:14. Al consultar (13:49) llevaba 36 min sin una muestra nueva. Etapa N°5, Estanque Inferior y Etapa 1 al 4 tenían trama dentro de los últimos 10 minutos.</t>
-        </is>
-      </c>
-      <c r="B37" s="19" t="n"/>
-      <c r="C37" s="19" t="n"/>
-      <c r="D37" s="19" t="n"/>
-      <c r="E37" s="19" t="n"/>
-      <c r="F37" s="19" t="n"/>
-      <c r="G37" s="19" t="n"/>
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>La Matriz ESVAL quedó en la trama de las 13:14. Al consultar (14:25) llevaba 12 min sin una muestra nueva. Etapa N°5, Estanque Inferior y Etapa 1 al 4 tenían trama dentro de los últimos 10 minutos.</t>
+        </is>
+      </c>
+      <c r="B37" s="69" t="n"/>
+      <c r="C37" s="69" t="n"/>
+      <c r="D37" s="69" t="n"/>
+      <c r="E37" s="69" t="n"/>
+      <c r="F37" s="69" t="n"/>
+      <c r="G37" s="70" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:C22"/>
@@ -1402,7 +1772,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00548235"/>
@@ -1694,12 +2064,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>015316</t>
+          <t>005316</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>365430</t>
+          <t>385430</t>
         </is>
       </c>
     </row>
@@ -1744,10 +2114,10 @@
         </is>
       </c>
       <c r="B22" s="21" t="n">
-        <v>15316.8</v>
+        <v>5316.8</v>
       </c>
       <c r="C22" s="21" t="n">
-        <v>365430.85</v>
+        <v>385430.8</v>
       </c>
     </row>
   </sheetData>
@@ -1769,14 +2139,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2077,43 +2447,60 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D19" s="23" t="n">
+        <v>0.08156606851549755</v>
+      </c>
+      <c r="E19" s="24" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Suma de horas</t>
         </is>
       </c>
-      <c r="B19" s="37">
-        <f>SUM(B5:B18)</f>
+      <c r="B20" s="37">
+        <f>SUM(B5:B19)</f>
         <v/>
       </c>
-      <c r="C19" s="37">
-        <f>SUM(C5:C18)</f>
+      <c r="C20" s="37">
+        <f>SUM(C5:C19)</f>
         <v/>
       </c>
-      <c r="D19" s="38">
-        <f>IF(B19=0,"—",C19/B19)</f>
+      <c r="D20" s="38">
+        <f>IF(B20=0,"—",C20/B20)</f>
         <v/>
       </c>
-      <c r="E19" s="39" t="inlineStr">
+      <c r="E20" s="39" t="inlineStr">
         <is>
           <t>Cierra con el total diario de la API</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>Total diario API: Matriz ESVAL 133,47 m³ · Etapa N°5 9,80 m³. El día sigue abierto: la hora 13 está incompleta y, en la Matriz, sin muestras desde las 13:14.</t>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Total diario API: Matriz ESVAL 139,60 m³ · Etapa N°5 10,30 m³. El día sigue abierto: la hora 13 está incompleta y, en la Matriz, sin muestras desde las 13:14.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E18"/>
+  <autoFilter ref="A4:E19"/>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A22:E22"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A21:E21"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
@@ -2128,7 +2515,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C65911"/>
@@ -2585,19 +2972,19 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>328.1</v>
+        <v>334.23</v>
       </c>
       <c r="C21" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="E21" s="12" t="n">
         <v>2</v>
       </c>
       <c r="F21" s="23" t="n">
-        <v>0.09753124047546478</v>
+        <v>0.09723842862699338</v>
       </c>
       <c r="G21" s="6" t="inlineStr"/>
     </row>
@@ -2672,7 +3059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -2775,10 +3162,10 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>15316.8</v>
+        <v>5316.8</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>365430.85</v>
+        <v>385430.8</v>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
@@ -2793,10 +3180,10 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>32268.48</v>
+        <v>32268.98</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>54428.66</v>
+        <v>54434.79</v>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
@@ -2829,10 +3216,10 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>14395.08</v>
+        <v>14395.58</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>52441.61</v>
+        <v>52447.74</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
@@ -2847,10 +3234,10 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>-16951.68</v>
+        <v>-26952.18</v>
       </c>
       <c r="C11" s="30" t="n">
-        <v>311002.19</v>
+        <v>330996.01</v>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
@@ -2865,10 +3252,10 @@
         </is>
       </c>
       <c r="B12" s="30" t="n">
-        <v>921.72</v>
+        <v>-9078.780000000001</v>
       </c>
       <c r="C12" s="30" t="n">
-        <v>312989.24</v>
+        <v>332983.06</v>
       </c>
       <c r="D12" s="54" t="inlineStr">
         <is>
@@ -2886,21 +3273,21 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Etapa N°5. El histórico completo de WES (32.268,5 m³) supera el dial (15.316,8 m³) en 16.951,7 m³. Eso lo explica marzo 2026: Etapa 5 marca 17.873,4 m³ y la Matriz 1.987,0 m³. Sin ese mes, WES suma 14.395,1 m³ y el dial le lleva 921,7 m³ (6,0% del dial). Esa diferencia cabe en el volumen anterior al monitoreo.</t>
+          <t>Etapa N°5. El histórico completo de WES (32.269,0 m³) supera el dial (5.316,8 m³) en 26.952,2 m³. Eso lo explica marzo 2026: Etapa 5 marca 17.873,4 m³ y la Matriz 1.987,0 m³. Sin ese mes, WES igual suma 14.395,6 m³, por encima del dial (5.316,8 m³). La comparación que cierra es la de relojería del 23-09 al 02-10, en la hoja Relojería.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Matriz ESVAL. El dial (365.430,85 m³) menos lo integrado por WES (54.428,7 m³) deja 311.002 m³ como índice al inicio de la serie (2025-06-25). Es el orden de un medidor de sanitaria que ya llevaba años instalado. Este cierre no confirma ni descarta el desfase entre m³ y L/min de hoy.</t>
+          <t>Matriz ESVAL. El dial (385.430,80 m³) menos lo integrado por WES (54.434,8 m³) deja 330.996 m³ como índice al inicio de la serie (2025-06-25). Es el orden de un medidor de sanitaria que ya llevaba años instalado. Este cierre no confirma ni descarta el desfase entre m³ y L/min de hoy.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Para cerrar el factor de la Matriz hace falta una segunda foto del mismo Flostar, con varias horas o un día de por medio, y restarla de esta lectura. Esa diferencia se compara con los m³ que sume WES entre las dos horas.</t>
+          <t>La segunda lectura ya está: la foto del 23-09-2026 del informe (Itron 384.148,9 m³ a las 17:05 y Sensus 5.177 m³ a las 16:54). La diferencia de relojería contra hoy se compara con la app en la hoja Relojería, con la misma regla de horas completas del informe del 23–28/09.</t>
         </is>
       </c>
     </row>
@@ -2939,17 +3326,15 @@
           <t>Ritmo del acumulado de m³</t>
         </is>
       </c>
-      <c r="B21" s="34" t="n">
-        <v>19.01</v>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="B21" s="34" t="n"/>
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>m³/h</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>De 0.800 m³ a las 13:03:14 a 3.680 m³ a las 13:12:20</t>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Sin muestras en la ventana</t>
         </is>
       </c>
     </row>
@@ -2960,16 +3345,16 @@
         </is>
       </c>
       <c r="B22" s="34" t="n">
-        <v>98</v>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
+        <v>100.86</v>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>L/min</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>15 muestras</t>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>7 muestras</t>
         </is>
       </c>
     </row>
@@ -2979,15 +3364,13 @@
           <t>Equivalente del ritmo de m³</t>
         </is>
       </c>
-      <c r="B23" s="34" t="n">
-        <v>316.84</v>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="B23" s="34" t="n"/>
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>L/min</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>m³/h × 1000 / 60</t>
         </is>
@@ -2999,29 +3382,27 @@
           <t>Veces que el canal de m³ supera al de L/min</t>
         </is>
       </c>
-      <c r="B24" s="34" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="B24" s="34" t="n"/>
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>veces</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Misma trama, dos canales</t>
         </is>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>Etapa N°5 en la hora 13 avanza en escalones de 0,1 m³ (0.0, 0.1, 0.2, 0.3, 0.4). Ese escalón es el pulso de 100 L del HRI para DN 80–125.</t>
-        </is>
-      </c>
-      <c r="B26" s="56" t="n"/>
-      <c r="C26" s="56" t="n"/>
-      <c r="D26" s="56" t="n"/>
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Etapa N°5 en la hora 13 avanza en escalones de 0,1 m³ (0.4, 0.5). Ese escalón es el pulso de 100 L del HRI para DN 80–125.</t>
+        </is>
+      </c>
+      <c r="B26" s="69" t="n"/>
+      <c r="C26" s="69" t="n"/>
+      <c r="D26" s="70" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3047,7 +3428,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>
@@ -3113,29 +3494,29 @@
           <t>Validado</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>La foto 1 es el Sensus MeiStream Plus 100 de Etapa N°5 (000027-03). Lectura 15.316,8 m³ a las 08:44. El punto seguía en línea a las 13:49 (0 L/min). El contador de WES sube de 0,1 en 0,1 m³, igual que el HRI de 100 L.</t>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>La foto de hoy es el mismo Sensus del informe (serie SEN01 2370 9030). El 23-09-2026 a las 16:54 el odómetro marcaba 5.177 m³. Hoy a las 08:44 marca 5.316,8 m³. El punto seguía en línea a las 14:25.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1">
-      <c r="A6" s="29" t="n">
+      <c r="A6" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="53" t="inlineStr">
+      <c r="B6" s="55" t="inlineStr">
         <is>
           <t>Etapa N°5</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
-        <is>
-          <t>Índice coherente</t>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>Relojería vs app</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Sin marzo 2026, WES suma 14.395,1 m³ desde 2025-06-25. El dial marca 15.316,8 m³: quedan 921,7 m³ (6,0% del dial) para el volumen previo al monitoreo.</t>
+          <t>Del 23-09 17:00 al 02-10 08:00 (hora de la foto excluida) la relojería avanza 139,8 m³ y la app suma 195,6 m³. Error 28,5 % (1 − 139,8/195,6). En la ventana 23–28/09 ese mismo medidor había cerrado en 0,8 %. El desvío aparece después del 28-09.</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3536,7 @@
       </c>
       <c r="D7" s="57" t="inlineStr">
         <is>
-          <t>En marzo 2026 Etapa N°5 marca 17.873,4 m³ y la Matriz 1.987,0 m³. Con ese mes, el histórico de WES (32.268,5 m³) supera toda la vida del medidor. Mayo 2026 también queda parejo con la Matriz (Etapa 5 un poco por encima) y conviene mirarlo aparte.</t>
+          <t>En marzo 2026 Etapa N°5 marca 17.873,4 m³ y la Matriz 1.987,0 m³. Con ese mes, el histórico de WES (32.269,0 m³) supera toda la vida del medidor. Mayo 2026 también queda parejo con la Matriz (Etapa 5 un poco por encima) y conviene mirarlo aparte.</t>
         </is>
       </c>
     </row>
@@ -3173,9 +3554,9 @@
           <t>Medidor identificado</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>La foto 2 es el Itron Flostar S de la Matriz ESVAL (000027-01), en Los Portones 378. Lectura 365.430,85 m³ a las 13:22. El índice al inicio de la serie WES queda cerca de 311.002 m³, propio de un medidor de sanitaria con años de servicio.</t>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>La foto de hoy es el mismo Itron Flostar S del informe, en Los Portones 378. El 23-09-2026 a las 17:05 marcaba 384.148,9 m³. Hoy a las 13:22 marca 385.430,8 m³. Relojería 1.281,9 m³ contra app 1.309,6 m³: error 2,1 %, del mismo orden que el 3,7 % del 23–28/09.</t>
         </is>
       </c>
     </row>
@@ -3195,7 +3576,7 @@
       </c>
       <c r="D9" s="57" t="inlineStr">
         <is>
-          <t>Última trama 021026 13:14. La foto es de las 13:22, con el punto ya mudo. A las 13:49 llevaba 36 min sin muestras. Etapa N°5, Estanque Inferior y Etapa 1 al 4 tenían trama dentro de los últimos 10 minutos.</t>
+          <t>Última trama 021026 14:14. La foto es de las 13:22, con el punto ya mudo. A las 14:25 llevaba 12 min sin muestras. Etapa N°5, Estanque Inferior y Etapa 1 al 4 tenían trama dentro de los últimos 10 minutos.</t>
         </is>
       </c>
     </row>
@@ -3213,9 +3594,9 @@
           <t>m³ y L/min no cierran</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>Entre 13:03 y 13:12 el acumulado de m³ subía a 19,0 m³/h (317 L/min) y los litros por minuto de la misma trama promediaban 98 L/min. El canal de m³ va 3,2 veces por encima. Con una sola foto no se sabe cuál de los dos canales está bien.</t>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>No hubo muestras suficientes para recalcular el desfase en esta consulta. Con una sola foto no se sabe cuál de los dos canales está bien.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use 5,174 m³ at 04:54 on 23 September as the Etapa 5 opening reading.
Recalculates the register difference against the complete-hour WES sum from 05:00 that day.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -997,7 +997,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="60" t="inlineStr">
         <is>
-          <t>Fotos de inicio rescatadas del informe de validación (23-09-2026). La app suma las horas completas del CSV, con la marca TIME en hora Chile, y deja fuera la hora de la foto final. Es la misma regla del cierre 23–28/09.</t>
+          <t>Fotos de inicio rescatadas del informe de validación (23-09-2026). Etapa N°5 parte en 5.174 m³ a las 04:54. La app suma las horas completas del CSV, con la marca TIME en hora Chile, y deja fuera la hora de cada foto.</t>
         </is>
       </c>
     </row>
@@ -1060,11 +1060,11 @@
         </is>
       </c>
       <c r="B5" s="62" t="n">
-        <v>5177</v>
+        <v>5174</v>
       </c>
       <c r="C5" s="63" t="inlineStr">
         <is>
-          <t>23-09-2026 16:54</t>
+          <t>23-09-2026 04:54</t>
         </is>
       </c>
       <c r="D5" s="62" t="n">
@@ -1076,16 +1076,16 @@
         </is>
       </c>
       <c r="F5" s="62" t="n">
-        <v>139.8000000000002</v>
+        <v>142.8</v>
       </c>
       <c r="G5" s="62" t="n">
-        <v>195.6</v>
+        <v>213.6</v>
       </c>
       <c r="H5" s="64" t="n">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="I5" s="35" t="n">
-        <v>0.2852760736196309</v>
+        <v>0.3314606741573033</v>
       </c>
       <c r="J5" s="33" t="inlineStr">
         <is>
@@ -1139,20 +1139,20 @@
           <t>Estanque Inferior en la misma ventana de la Matriz: 1.133,4 m³ (87 % de la app, 212 horas). En el cierre 23–28/09 ese porcentaje era 87 %.</t>
         </is>
       </c>
-      <c r="B7" s="68" t="n"/>
-      <c r="C7" s="68" t="n"/>
-      <c r="D7" s="68" t="n"/>
-      <c r="E7" s="68" t="n"/>
-      <c r="F7" s="68" t="n"/>
-      <c r="G7" s="68" t="n"/>
-      <c r="H7" s="68" t="n"/>
-      <c r="I7" s="68" t="n"/>
-      <c r="J7" s="68" t="n"/>
+      <c r="B7" s="69" t="n"/>
+      <c r="C7" s="69" t="n"/>
+      <c r="D7" s="69" t="n"/>
+      <c r="E7" s="69" t="n"/>
+      <c r="F7" s="69" t="n"/>
+      <c r="G7" s="69" t="n"/>
+      <c r="H7" s="69" t="n"/>
+      <c r="I7" s="69" t="n"/>
+      <c r="J7" s="70" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Etapa N°5. El 23–28/09 este Sensus cerró en 0,8 % (48 m³ de relojería contra 47,6 m³ de app). Del 23-09 al 02-10 la app queda 55,8 m³ por encima de la relojería. El desvío es posterior al 28-09.</t>
+          <t>Etapa N°5. Lectura inicial 5.174 m³ a las 04:54 del 23-09. Hoy 5.316,8 m³ a las 08:44. Relojería 142,8 m³ contra app 213,6 m³ (error 33,1 %). La suma parte a las 05:00, la hora siguiente a la foto, y deja fuera las 08:00 del 02-10. La hora 04 del 23-09 en la app es 0,00 m³.</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>005316 m³; décima girando de 8 a 9. Mismo odómetro que el 5.177 del 23-09</t>
+          <t>005316 m³; décima girando de 8 a 9. Mismo odómetro que el 5.174 del 23-09 a las 04:54</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Odómetro 005316,8. Contra el 5.177 del 23-09 la relojería avanza 139,8 m³ y la app suma 195,6 m³.</t>
+          <t>Odómetro 005316,8. Contra el 5.174 de las 04:54 del 23-09 la relojería avanza 142,8 m³ y la app suma 213,6 m³.</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1531,7 +1531,7 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Etapa N°5: el mismo Sensus del informe del 23-09 (odómetro 005177). Hoy los rodillos marcan 005316 y la décima está entre 8 y 9. Se registra 5.316,8 m³.</t>
+          <t>Etapa N°5: lectura inicial 5.174 m³ a las 04:54 del 23-09. Hoy los rodillos marcan 005316 y la décima está entre 8 y 9. Se registra 5.316,8 m³.</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>La segunda lectura ya está: la foto del 23-09-2026 del informe (Itron 384.148,9 m³ a las 17:05 y Sensus 5.177 m³ a las 16:54). La diferencia de relojería contra hoy se compara con la app en la hoja Relojería, con la misma regla de horas completas del informe del 23–28/09.</t>
+          <t>La lectura inicial de Etapa N°5 es 5.174 m³ a las 04:54 del 23-09. La Matriz parte en el Itron del mismo informe: 384.148,9 m³ a las 17:05. La diferencia de relojería contra hoy está en la hoja Relojería.</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>La foto de hoy es el mismo Sensus del informe (serie SEN01 2370 9030). El 23-09-2026 a las 16:54 el odómetro marcaba 5.177 m³. Hoy a las 08:44 marca 5.316,8 m³. El punto seguía en línea a las 14:25.</t>
+          <t>La foto de hoy es el mismo Sensus del informe (serie SEN01 2370 9030). La lectura inicial es 5.174 m³ a las 04:54 del 23-09. Hoy a las 08:44 marca 5.316,8 m³.</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3516,7 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Del 23-09 17:00 al 02-10 08:00 (hora de la foto excluida) la relojería avanza 139,8 m³ y la app suma 195,6 m³. Error 28,5 % (1 − 139,8/195,6). En la ventana 23–28/09 ese mismo medidor había cerrado en 0,8 %. El desvío aparece después del 28-09.</t>
+          <t>Del 23-09 05:00 al 02-10 08:00 (horas de las fotos fuera de la suma) la relojería avanza 142,8 m³ y la app suma 213,6 m³. Error 33,1 % (1 − 142,8/213,6). 219 horas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct the Friday Etapa 5 reading to 5,369 m³.
The 2 October photo was stored as 5,316.8 m³. With 5,369 m³ the register advances 195.0 m³ against 213.6 m³ in the app from 23 September 05:00, and 144 m³ against 148.0 m³ after the 28 September photo.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relojeria" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lecturas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horario hoy" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historico mensual" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cierre de indice" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hallazgos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Relojeria" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lecturas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Horario hoy" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Historico mensual" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cierre de indice" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Hallazgos" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relojeria'!$A$4:$J$6</definedName>
@@ -219,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -403,6 +403,21 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,13 +495,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -510,7 +525,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -534,7 +549,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -573,8 +588,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -601,7 +616,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -616,13 +631,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -641,13 +656,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -656,7 +671,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -671,9 +686,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1068,7 +1083,7 @@
         </is>
       </c>
       <c r="D5" s="62" t="n">
-        <v>5316.8</v>
+        <v>5369</v>
       </c>
       <c r="E5" s="63" t="inlineStr">
         <is>
@@ -1076,7 +1091,7 @@
         </is>
       </c>
       <c r="F5" s="62" t="n">
-        <v>142.8</v>
+        <v>195</v>
       </c>
       <c r="G5" s="62" t="n">
         <v>213.6</v>
@@ -1085,7 +1100,7 @@
         <v>219</v>
       </c>
       <c r="I5" s="35" t="n">
-        <v>0.3314606741573033</v>
+        <v>0.08707865168539319</v>
       </c>
       <c r="J5" s="33" t="inlineStr">
         <is>
@@ -1149,10 +1164,10 @@
       <c r="I7" s="69" t="n"/>
       <c r="J7" s="70" t="n"/>
     </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Etapa N°5. Lectura inicial 5.174 m³ a las 04:54 del 23-09. Hoy 5.316,8 m³ a las 08:44. Relojería 142,8 m³ contra app 213,6 m³ (error 33,1 %). La suma parte a las 05:00, la hora siguiente a la foto, y deja fuera las 08:00 del 02-10. La hora 04 del 23-09 en la app es 0,00 m³.</t>
+    <row r="9" ht="62" customHeight="1">
+      <c r="A9" s="71" t="inlineStr">
+        <is>
+          <t>Etapa N°5. Lectura inicial 5.174 m³ a las 04:54 del 23-09. El viernes 02-10 a las 08:44 marca 5.369 m³ (la versión anterior decía 5.316,8: el 6 y el 9 se leyeron al revés). Relojería 195,0 m³ contra app 213,6 m³ (error 8,7 %). La suma parte a las 05:00 y deja fuera las 08:00 del 02-10. Desde la foto del 28-09 (5.225 m³ a las 08:57) hasta el viernes la relojería avanza 144 m³ y la app 148,0 m³ (error 2,7 %): ese tramo cierra. La hora impresa en la foto del 23-09 es 16:54; con esa hora la app suma 195,6 m³ y el error baja a 0,3 %.</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1410,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>5316.8</v>
+        <v>5369</v>
       </c>
       <c r="C14" s="7" t="n">
         <v>385430.8</v>
@@ -1407,9 +1422,9 @@
           <t>Detalle de la lectura</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>005316 m³; décima girando de 8 a 9. Mismo odómetro que el 5.174 del 23-09 a las 04:54</t>
+      <c r="B15" s="72" t="inlineStr">
+        <is>
+          <t>005369 m³. Mismo odómetro que el 5.174 del 23-09 a las 04:54. La lectura anterior 5.316,8 cambió el 6 por un 1 y el 9 por un 6.</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1510,9 +1525,9 @@
           <t>Lectura de la validación</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Odómetro 005316,8. Contra el 5.174 de las 04:54 del 23-09 la relojería avanza 142,8 m³ y la app suma 213,6 m³.</t>
+      <c r="B22" s="73" t="inlineStr">
+        <is>
+          <t>Odómetro 5.369. Contra el 5.174 de las 04:54 del 23-09 la relojería avanza 195,0 m³ y la app suma 213,6 m³.</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1529,9 +1544,9 @@
       </c>
     </row>
     <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>Etapa N°5: lectura inicial 5.174 m³ a las 04:54 del 23-09. Hoy los rodillos marcan 005316 y la décima está entre 8 y 9. Se registra 5.316,8 m³.</t>
+      <c r="A25" s="71" t="inlineStr">
+        <is>
+          <t>Etapa N°5: lectura inicial 5.174 m³ a las 04:54 del 23-09. El viernes 02-10 los rodillos marcan 005369. Se registra 5.369 m³.</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2079,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>005316</t>
+          <t>005369</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -2081,7 +2096,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Décima entre 8 y 9</t>
+          <t>Último rodillo en 9</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -2114,7 +2129,7 @@
         </is>
       </c>
       <c r="B22" s="21" t="n">
-        <v>5316.8</v>
+        <v>5369</v>
       </c>
       <c r="C22" s="21" t="n">
         <v>385430.8</v>
@@ -3162,7 +3177,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>5316.8</v>
+        <v>5369</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>385430.8</v>
@@ -3234,7 +3249,7 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>-26952.18</v>
+        <v>-26899.98</v>
       </c>
       <c r="C11" s="30" t="n">
         <v>330996.01</v>
@@ -3252,7 +3267,7 @@
         </is>
       </c>
       <c r="B12" s="30" t="n">
-        <v>-9078.780000000001</v>
+        <v>-9026.58</v>
       </c>
       <c r="C12" s="30" t="n">
         <v>332983.06</v>
@@ -3271,9 +3286,9 @@
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>Etapa N°5. El histórico completo de WES (32.269,0 m³) supera el dial (5.316,8 m³) en 26.952,2 m³. Eso lo explica marzo 2026: Etapa 5 marca 17.873,4 m³ y la Matriz 1.987,0 m³. Sin ese mes, WES igual suma 14.395,6 m³, por encima del dial (5.316,8 m³). La comparación que cierra es la de relojería del 23-09 al 02-10, en la hoja Relojería.</t>
+      <c r="A15" s="71" t="inlineStr">
+        <is>
+          <t>Etapa N°5. El histórico completo de WES (32.269,0 m³) supera el dial (5.369 m³) en 26.900,0 m³. Eso lo explica marzo 2026: Etapa 5 marca 17.873,4 m³ y la Matriz 1.987,0 m³. Sin ese mes, WES igual suma 14.395,6 m³, por encima del dial (5.369 m³). La comparación que cierra es la de relojería del 23-09 al 02-10, en la hoja Relojería.</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3495,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="62" customHeight="1">
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="29" t="n">
         <v>1</v>
       </c>
@@ -3494,9 +3509,9 @@
           <t>Validado</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>La foto de hoy es el mismo Sensus del informe (serie SEN01 2370 9030). La lectura inicial es 5.174 m³ a las 04:54 del 23-09. Hoy a las 08:44 marca 5.316,8 m³.</t>
+      <c r="D5" s="74" t="inlineStr">
+        <is>
+          <t>La foto del viernes 02-10 es el mismo Sensus del informe (serie SEN01 2370 9030). La lectura inicial es 5.174 m³ a las 04:54 del 23-09. El viernes a las 08:44 marca 5.369 m³. La cifra 5.316,8 salió de leer el 6 como 1 y el 9 como 6.</t>
         </is>
       </c>
     </row>
@@ -3514,9 +3529,9 @@
           <t>Relojería vs app</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Del 23-09 05:00 al 02-10 08:00 (horas de las fotos fuera de la suma) la relojería avanza 142,8 m³ y la app suma 213,6 m³. Error 33,1 % (1 − 142,8/213,6). 219 horas.</t>
+      <c r="D6" s="75" t="inlineStr">
+        <is>
+          <t>Del 23-09 05:00 al 02-10 08:00 (horas de las fotos fuera de la suma) la relojería avanza 195,0 m³ y la app suma 213,6 m³. Error 8,7 % (1 − 195,0/213,6). 219 horas. Desde el 28-09 08:57 (5.225 m³) hasta el viernes la relojería avanza 144 m³ y la app 148,0 m³ (error 2,7 %): ese tramo cierra. Con la hora impresa en la foto del 23-09 (16:54) la app suma 195,6 m³ y el error es 0,3 %.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use 16:54 on 23 September as the Etapa 5 opening time.
The 5,174 m³ reading is at 16:54. From 17:00 that day to 08:00 on 2 October the register advances 195.0 m³ and the app sums 195.6 m³, an error of 0.3% over 207 hours.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -219,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -417,6 +417,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1010,9 +1013,9 @@
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="60" t="inlineStr">
-        <is>
-          <t>Fotos de inicio rescatadas del informe de validación (23-09-2026). Etapa N°5 parte en 5.174 m³ a las 04:54. La app suma las horas completas del CSV, con la marca TIME en hora Chile, y deja fuera la hora de cada foto.</t>
+      <c r="A2" s="76" t="inlineStr">
+        <is>
+          <t>Fotos de inicio rescatadas del informe de validación (23-09-2026). Etapa N°5 parte en 5.174 m³ a las 16:54. La app suma las horas completas del CSV, con la marca TIME en hora Chile, y deja fuera la hora de cada foto.</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1082,7 @@
       </c>
       <c r="C5" s="63" t="inlineStr">
         <is>
-          <t>23-09-2026 04:54</t>
+          <t>23-09-2026 16:54</t>
         </is>
       </c>
       <c r="D5" s="62" t="n">
@@ -1094,17 +1097,17 @@
         <v>195</v>
       </c>
       <c r="G5" s="62" t="n">
-        <v>213.6</v>
+        <v>195.6</v>
       </c>
       <c r="H5" s="64" t="n">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="I5" s="35" t="n">
-        <v>0.08707865168539319</v>
+        <v>0.003067484662576669</v>
       </c>
       <c r="J5" s="33" t="inlineStr">
         <is>
-          <t>Revisar</t>
+          <t>Aceptable</t>
         </is>
       </c>
     </row>
@@ -1164,10 +1167,10 @@
       <c r="I7" s="69" t="n"/>
       <c r="J7" s="70" t="n"/>
     </row>
-    <row r="9" ht="62" customHeight="1">
+    <row r="9" ht="52" customHeight="1">
       <c r="A9" s="71" t="inlineStr">
         <is>
-          <t>Etapa N°5. Lectura inicial 5.174 m³ a las 04:54 del 23-09. El viernes 02-10 a las 08:44 marca 5.369 m³ (la versión anterior decía 5.316,8: el 6 y el 9 se leyeron al revés). Relojería 195,0 m³ contra app 213,6 m³ (error 8,7 %). La suma parte a las 05:00 y deja fuera las 08:00 del 02-10. Desde la foto del 28-09 (5.225 m³ a las 08:57) hasta el viernes la relojería avanza 144 m³ y la app 148,0 m³ (error 2,7 %): ese tramo cierra. La hora impresa en la foto del 23-09 es 16:54; con esa hora la app suma 195,6 m³ y el error baja a 0,3 %.</t>
+          <t>Etapa N°5. Lectura inicial 5.174 m³ a las 16:54 del 23-09. El viernes 02-10 a las 08:44 marca 5.369 m³. Relojería 195,0 m³ contra app 195,6 m³ (error 0,3 %). La suma parte a las 17:00, la hora siguiente a la foto, y deja fuera las 08:00 del 02-10. 207 horas. Desde la foto del 28-09 (5.225 m³ a las 08:57) hasta el viernes la relojería avanza 144 m³ y la app 148,0 m³ (error 2,7 %).</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1427,7 @@
       </c>
       <c r="B15" s="72" t="inlineStr">
         <is>
-          <t>005369 m³. Mismo odómetro que el 5.174 del 23-09 a las 04:54. La lectura anterior 5.316,8 cambió el 6 por un 1 y el 9 por un 6.</t>
+          <t>005369 m³. Mismo odómetro que el 5.174 del 23-09 a las 16:54.</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1527,7 +1530,7 @@
       </c>
       <c r="B22" s="73" t="inlineStr">
         <is>
-          <t>Odómetro 5.369. Contra el 5.174 de las 04:54 del 23-09 la relojería avanza 195,0 m³ y la app suma 213,6 m³.</t>
+          <t>Odómetro 5.369. Contra el 5.174 de las 16:54 del 23-09 la relojería avanza 195,0 m³ y la app suma 195,6 m³.</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1546,7 +1549,7 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="71" t="inlineStr">
         <is>
-          <t>Etapa N°5: lectura inicial 5.174 m³ a las 04:54 del 23-09. El viernes 02-10 los rodillos marcan 005369. Se registra 5.369 m³.</t>
+          <t>Etapa N°5: lectura inicial 5.174 m³ a las 16:54 del 23-09. El viernes 02-10 los rodillos marcan 005369. Se registra 5.369 m³.</t>
         </is>
       </c>
     </row>
@@ -3300,9 +3303,9 @@
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>La lectura inicial de Etapa N°5 es 5.174 m³ a las 04:54 del 23-09. La Matriz parte en el Itron del mismo informe: 384.148,9 m³ a las 17:05. La diferencia de relojería contra hoy está en la hoja Relojería.</t>
+      <c r="A17" s="71" t="inlineStr">
+        <is>
+          <t>La lectura inicial de Etapa N°5 es 5.174 m³ a las 16:54 del 23-09. La Matriz parte en el Itron del mismo informe: 384.148,9 m³ a las 17:05. La diferencia de relojería contra hoy está en la hoja Relojería.</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3514,7 @@
       </c>
       <c r="D5" s="74" t="inlineStr">
         <is>
-          <t>La foto del viernes 02-10 es el mismo Sensus del informe (serie SEN01 2370 9030). La lectura inicial es 5.174 m³ a las 04:54 del 23-09. El viernes a las 08:44 marca 5.369 m³. La cifra 5.316,8 salió de leer el 6 como 1 y el 9 como 6.</t>
+          <t>La foto del viernes 02-10 es el mismo Sensus del informe (serie SEN01 2370 9030). La lectura inicial es 5.174 m³ a las 16:54 del 23-09. El viernes a las 08:44 marca 5.369 m³.</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3534,7 @@
       </c>
       <c r="D6" s="75" t="inlineStr">
         <is>
-          <t>Del 23-09 05:00 al 02-10 08:00 (horas de las fotos fuera de la suma) la relojería avanza 195,0 m³ y la app suma 213,6 m³. Error 8,7 % (1 − 195,0/213,6). 219 horas. Desde el 28-09 08:57 (5.225 m³) hasta el viernes la relojería avanza 144 m³ y la app 148,0 m³ (error 2,7 %): ese tramo cierra. Con la hora impresa en la foto del 23-09 (16:54) la app suma 195,6 m³ y el error es 0,3 %.</t>
+          <t>Del 23-09 17:00 al 02-10 08:00 (horas de las fotos fuera de la suma) la relojería avanza 195,0 m³ y la app suma 195,6 m³. Error 0,3 % (1 − 195,0/195,6). 207 horas. Desde el 28-09 08:57 (5.225 m³) hasta el viernes la relojería avanza 144 m³ y la app 148,0 m³ (error 2,7 %).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add app totals for the same 16:54 to 08:44 window.
Estanque Inferior, Etapa 5 and Etapa 1 al 4 are summed on complete hours from 23 September 17:00 through 2 October 07:00.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -8,27 +8,30 @@
   </bookViews>
   <sheets>
     <sheet name="Relojeria" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lecturas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Horario hoy" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Historico mensual" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Cierre de indice" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Hallazgos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Misma ventana" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lecturas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Horario hoy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Historico mensual" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cierre de indice" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Hallazgos" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relojeria'!$A$4:$J$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Relojeria'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resumen'!$A$5:$C$22</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Resumen'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lecturas'!$A$4:$C$22</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Lecturas'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Horario hoy'!$A$4:$E$19</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Horario hoy'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Historico mensual'!$A$4:$G$21</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Historico mensual'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Cierre de indice'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Hallazgos'!$A$4:$D$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Hallazgos'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Misma ventana'!$A$4:$E$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Misma ventana'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resumen'!$A$5:$C$22</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Resumen'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lecturas'!$A$4:$C$22</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lecturas'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Horario hoy'!$A$4:$E$19</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Horario hoy'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Historico mensual'!$A$4:$G$21</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Historico mensual'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Cierre de indice'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Hallazgos'!$A$4:$D$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Hallazgos'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -39,7 +42,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,6 +98,23 @@
       <color rgb="001F4E79"/>
       <sz val="18"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00334155"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -149,7 +169,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -215,11 +235,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D7DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D7DE"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -421,6 +455,28 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -641,6 +697,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -666,6 +725,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1216,6 +1278,356 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>App WES en la misma ventana de Etapa N°5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="78" t="inlineStr">
+        <is>
+          <t>Del 23-09-2026 16:54 al 02-10-2026 08:44. La suma usa horas completas: desde las 17:00 del 23-09 hasta antes de las 08:00 del 02-10. La marca TIME está en hora Chile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="79" t="inlineStr">
+        <is>
+          <t>Punto</t>
+        </is>
+      </c>
+      <c r="B4" s="79" t="inlineStr">
+        <is>
+          <t>Nodo</t>
+        </is>
+      </c>
+      <c r="C4" s="79" t="inlineStr">
+        <is>
+          <t>App WES (m³)</t>
+        </is>
+      </c>
+      <c r="D4" s="79" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="E4" s="79" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="80" t="inlineStr">
+        <is>
+          <t>Estanque Inferior</t>
+        </is>
+      </c>
+      <c r="B5" s="81" t="inlineStr">
+        <is>
+          <t>000027-02</t>
+        </is>
+      </c>
+      <c r="C5" s="82" t="n">
+        <v>1100.1</v>
+      </c>
+      <c r="D5" s="81" t="n">
+        <v>207</v>
+      </c>
+      <c r="E5" s="81" t="inlineStr">
+        <is>
+          <t>207 horas completas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="80" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="B6" s="81" t="inlineStr">
+        <is>
+          <t>000027-03</t>
+        </is>
+      </c>
+      <c r="C6" s="82" t="n">
+        <v>195.6</v>
+      </c>
+      <c r="D6" s="81" t="n">
+        <v>207</v>
+      </c>
+      <c r="E6" s="81" t="inlineStr">
+        <is>
+          <t>Misma ventana de la relojería 5.174 → 5.369 m³</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="80" t="inlineStr">
+        <is>
+          <t>Etapa 1 al 4</t>
+        </is>
+      </c>
+      <c r="B7" s="81" t="inlineStr">
+        <is>
+          <t>000027-04</t>
+        </is>
+      </c>
+      <c r="C7" s="82" t="n">
+        <v>725.58</v>
+      </c>
+      <c r="D7" s="81" t="n">
+        <v>206</v>
+      </c>
+      <c r="E7" s="81" t="inlineStr">
+        <is>
+          <t>Falta la hora 14:00 del 24-09; la suma es de las 206 horas con dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="83" t="inlineStr">
+        <is>
+          <t>m³ por día dentro de la ventana</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="84" t="inlineStr">
+        <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="B10" s="84" t="inlineStr">
+        <is>
+          <t>Estanque Inferior</t>
+        </is>
+      </c>
+      <c r="C10" s="84" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="D10" s="84" t="inlineStr">
+        <is>
+          <t>Etapa 1 al 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="85" t="inlineStr">
+        <is>
+          <t>23-09-2026 desde 17:00</t>
+        </is>
+      </c>
+      <c r="B11" s="86" t="n">
+        <v>18.26</v>
+      </c>
+      <c r="C11" s="86" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D11" s="86" t="n">
+        <v>8.01</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="85" t="inlineStr">
+        <is>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="B12" s="86" t="n">
+        <v>142.11</v>
+      </c>
+      <c r="C12" s="86" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="D12" s="86" t="n">
+        <v>81.48999999999999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="85" t="inlineStr">
+        <is>
+          <t>25-09-2026</t>
+        </is>
+      </c>
+      <c r="B13" s="86" t="n">
+        <v>128.52</v>
+      </c>
+      <c r="C13" s="86" t="n">
+        <v>13</v>
+      </c>
+      <c r="D13" s="86" t="n">
+        <v>90.23999999999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="85" t="inlineStr">
+        <is>
+          <t>26-09-2026</t>
+        </is>
+      </c>
+      <c r="B14" s="86" t="n">
+        <v>98.81</v>
+      </c>
+      <c r="C14" s="86" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D14" s="86" t="n">
+        <v>58.56</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="85" t="inlineStr">
+        <is>
+          <t>27-09-2026</t>
+        </is>
+      </c>
+      <c r="B15" s="86" t="n">
+        <v>82.17</v>
+      </c>
+      <c r="C15" s="86" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D15" s="86" t="n">
+        <v>66.52</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="85" t="inlineStr">
+        <is>
+          <t>28-09-2026</t>
+        </is>
+      </c>
+      <c r="B16" s="86" t="n">
+        <v>109.52</v>
+      </c>
+      <c r="C16" s="86" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="D16" s="86" t="n">
+        <v>72.23</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="85" t="inlineStr">
+        <is>
+          <t>29-09-2026</t>
+        </is>
+      </c>
+      <c r="B17" s="86" t="n">
+        <v>120.97</v>
+      </c>
+      <c r="C17" s="86" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="D17" s="86" t="n">
+        <v>80.69</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="85" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="B18" s="86" t="n">
+        <v>170.73</v>
+      </c>
+      <c r="C18" s="86" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="D18" s="86" t="n">
+        <v>106.17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="85" t="inlineStr">
+        <is>
+          <t>01-10-2026</t>
+        </is>
+      </c>
+      <c r="B19" s="86" t="n">
+        <v>158.2</v>
+      </c>
+      <c r="C19" s="86" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="D19" s="86" t="n">
+        <v>111.39</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="85" t="inlineStr">
+        <is>
+          <t>02-10-2026 hasta 07:00</t>
+        </is>
+      </c>
+      <c r="B20" s="86" t="n">
+        <v>70.81</v>
+      </c>
+      <c r="C20" s="86" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D20" s="86" t="n">
+        <v>50.28</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="87" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B21" s="88" t="n">
+        <v>1100.1</v>
+      </c>
+      <c r="C21" s="88" t="n">
+        <v>195.6</v>
+      </c>
+      <c r="D21" s="88" t="n">
+        <v>725.58</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:E7"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;LFundo Zapallar&amp;R23-09 16:54 a 02-10 08:44</oddHeader>
+    <oddFooter>&amp;LApp WES, horas completas&amp;RPágina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001F4788"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -1790,7 +2202,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00548235"/>
@@ -2157,7 +2569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
@@ -2533,7 +2945,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C65911"/>
@@ -3077,7 +3489,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -3446,7 +3858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>

</xml_diff>

<commit_message>
Add Matriz ESVAL and a total to the daily window table.
The same 16:54 to 08:44 window now lists Matriz ESVAL beside the other points, with a total of Estanque Inferior, Etapa 5 and Etapa 1 al 4.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -19,8 +19,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relojeria'!$A$4:$J$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Relojeria'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Misma ventana'!$A$4:$E$7</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Misma ventana'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Misma ventana'!$A$5:$F$15</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Misma ventana'!$1:$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resumen'!$A$5:$C$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Resumen'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lecturas'!$A$4:$C$22</definedName>
@@ -253,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -477,6 +477,25 @@
     <xf numFmtId="4" fontId="6" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1281,14 +1300,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1298,321 +1318,349 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="78" t="inlineStr">
         <is>
-          <t>Del 23-09-2026 16:54 al 02-10-2026 08:44. La suma usa horas completas: desde las 17:00 del 23-09 hasta antes de las 08:00 del 02-10. La marca TIME está en hora Chile.</t>
+          <t>Del 23-09-2026 16:54 al 02-10-2026 08:44. La suma usa horas completas: desde las 17:00 del 23-09 hasta antes de las 08:00 del 02-10. La marca TIME está en hora Chile. La columna Total suma Estanque Inferior, Etapa N°5 y Etapa 1 al 4.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="79" t="inlineStr">
-        <is>
-          <t>Punto</t>
-        </is>
-      </c>
-      <c r="B4" s="79" t="inlineStr">
-        <is>
-          <t>Nodo</t>
-        </is>
-      </c>
-      <c r="C4" s="79" t="inlineStr">
-        <is>
-          <t>App WES (m³)</t>
-        </is>
-      </c>
-      <c r="D4" s="79" t="inlineStr">
-        <is>
-          <t>Horas</t>
-        </is>
-      </c>
-      <c r="E4" s="79" t="inlineStr">
-        <is>
-          <t>Nota</t>
+      <c r="A4" s="83" t="inlineStr">
+        <is>
+          <t>m³ por día dentro de la ventana</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="80" t="inlineStr">
+      <c r="A5" s="89" t="inlineStr">
+        <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="B5" s="89" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL</t>
+        </is>
+      </c>
+      <c r="C5" s="89" t="inlineStr">
         <is>
           <t>Estanque Inferior</t>
         </is>
       </c>
-      <c r="B5" s="81" t="inlineStr">
-        <is>
-          <t>000027-02</t>
-        </is>
-      </c>
-      <c r="C5" s="82" t="n">
+      <c r="D5" s="89" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="E5" s="89" t="inlineStr">
+        <is>
+          <t>Etapa 1 al 4</t>
+        </is>
+      </c>
+      <c r="F5" s="89" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="90" t="inlineStr">
+        <is>
+          <t>23-09-2026 desde 17:00</t>
+        </is>
+      </c>
+      <c r="B6" s="91" t="n">
+        <v>24.17</v>
+      </c>
+      <c r="C6" s="91" t="n">
+        <v>18.26</v>
+      </c>
+      <c r="D6" s="91" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E6" s="91" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="F6" s="92" t="n">
+        <v>27.17</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="90" t="inlineStr">
+        <is>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="B7" s="91" t="n">
+        <v>161.76</v>
+      </c>
+      <c r="C7" s="91" t="n">
+        <v>142.11</v>
+      </c>
+      <c r="D7" s="91" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="E7" s="91" t="n">
+        <v>81.48999999999999</v>
+      </c>
+      <c r="F7" s="92" t="n">
+        <v>243.1</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="90" t="inlineStr">
+        <is>
+          <t>25-09-2026</t>
+        </is>
+      </c>
+      <c r="B8" s="91" t="n">
+        <v>148.61</v>
+      </c>
+      <c r="C8" s="91" t="n">
+        <v>128.52</v>
+      </c>
+      <c r="D8" s="91" t="n">
+        <v>13</v>
+      </c>
+      <c r="E8" s="91" t="n">
+        <v>90.23999999999999</v>
+      </c>
+      <c r="F8" s="92" t="n">
+        <v>231.76</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="90" t="inlineStr">
+        <is>
+          <t>26-09-2026</t>
+        </is>
+      </c>
+      <c r="B9" s="91" t="n">
+        <v>112.95</v>
+      </c>
+      <c r="C9" s="91" t="n">
+        <v>98.81</v>
+      </c>
+      <c r="D9" s="91" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E9" s="91" t="n">
+        <v>58.56</v>
+      </c>
+      <c r="F9" s="92" t="n">
+        <v>162.27</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="90" t="inlineStr">
+        <is>
+          <t>27-09-2026</t>
+        </is>
+      </c>
+      <c r="B10" s="91" t="n">
+        <v>95.09</v>
+      </c>
+      <c r="C10" s="91" t="n">
+        <v>82.17</v>
+      </c>
+      <c r="D10" s="91" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E10" s="91" t="n">
+        <v>66.52</v>
+      </c>
+      <c r="F10" s="92" t="n">
+        <v>153.59</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="90" t="inlineStr">
+        <is>
+          <t>28-09-2026</t>
+        </is>
+      </c>
+      <c r="B11" s="91" t="n">
+        <v>127.82</v>
+      </c>
+      <c r="C11" s="91" t="n">
+        <v>109.52</v>
+      </c>
+      <c r="D11" s="91" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="E11" s="91" t="n">
+        <v>72.23</v>
+      </c>
+      <c r="F11" s="92" t="n">
+        <v>201.05</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="90" t="inlineStr">
+        <is>
+          <t>29-09-2026</t>
+        </is>
+      </c>
+      <c r="B12" s="91" t="n">
+        <v>137.71</v>
+      </c>
+      <c r="C12" s="91" t="n">
+        <v>120.97</v>
+      </c>
+      <c r="D12" s="91" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="E12" s="91" t="n">
+        <v>80.69</v>
+      </c>
+      <c r="F12" s="92" t="n">
+        <v>255.76</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="90" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="B13" s="91" t="n">
+        <v>191.16</v>
+      </c>
+      <c r="C13" s="91" t="n">
+        <v>170.73</v>
+      </c>
+      <c r="D13" s="91" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="E13" s="91" t="n">
+        <v>106.17</v>
+      </c>
+      <c r="F13" s="92" t="n">
+        <v>329.5</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="90" t="inlineStr">
+        <is>
+          <t>01-10-2026</t>
+        </is>
+      </c>
+      <c r="B14" s="91" t="n">
+        <v>194.63</v>
+      </c>
+      <c r="C14" s="91" t="n">
+        <v>158.2</v>
+      </c>
+      <c r="D14" s="91" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="E14" s="91" t="n">
+        <v>111.39</v>
+      </c>
+      <c r="F14" s="92" t="n">
+        <v>291.79</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="90" t="inlineStr">
+        <is>
+          <t>02-10-2026 hasta 07:00</t>
+        </is>
+      </c>
+      <c r="B15" s="91" t="n">
+        <v>77.38</v>
+      </c>
+      <c r="C15" s="91" t="n">
+        <v>70.81</v>
+      </c>
+      <c r="D15" s="91" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E15" s="91" t="n">
+        <v>50.28</v>
+      </c>
+      <c r="F15" s="92" t="n">
+        <v>125.29</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="93" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B16" s="94" t="n">
+        <v>1271.28</v>
+      </c>
+      <c r="C16" s="94" t="n">
         <v>1100.1</v>
       </c>
-      <c r="D5" s="81" t="n">
-        <v>207</v>
-      </c>
-      <c r="E5" s="81" t="inlineStr">
-        <is>
-          <t>207 horas completas</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="80" t="inlineStr">
-        <is>
-          <t>Etapa N°5</t>
-        </is>
-      </c>
-      <c r="B6" s="81" t="inlineStr">
-        <is>
-          <t>000027-03</t>
-        </is>
-      </c>
-      <c r="C6" s="82" t="n">
+      <c r="D16" s="94" t="n">
         <v>195.6</v>
       </c>
-      <c r="D6" s="81" t="n">
-        <v>207</v>
-      </c>
-      <c r="E6" s="81" t="inlineStr">
-        <is>
-          <t>Misma ventana de la relojería 5.174 → 5.369 m³</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="80" t="inlineStr">
-        <is>
-          <t>Etapa 1 al 4</t>
-        </is>
-      </c>
-      <c r="B7" s="81" t="inlineStr">
-        <is>
-          <t>000027-04</t>
-        </is>
-      </c>
-      <c r="C7" s="82" t="n">
+      <c r="E16" s="94" t="n">
         <v>725.58</v>
       </c>
-      <c r="D7" s="81" t="n">
-        <v>206</v>
-      </c>
-      <c r="E7" s="81" t="inlineStr">
-        <is>
-          <t>Falta la hora 14:00 del 24-09; la suma es de las 206 horas con dato</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="83" t="inlineStr">
-        <is>
-          <t>m³ por día dentro de la ventana</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="84" t="inlineStr">
-        <is>
-          <t>Día</t>
-        </is>
-      </c>
-      <c r="B10" s="84" t="inlineStr">
-        <is>
-          <t>Estanque Inferior</t>
-        </is>
-      </c>
-      <c r="C10" s="84" t="inlineStr">
-        <is>
-          <t>Etapa N°5</t>
-        </is>
-      </c>
-      <c r="D10" s="84" t="inlineStr">
-        <is>
-          <t>Etapa 1 al 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="85" t="inlineStr">
-        <is>
-          <t>23-09-2026 desde 17:00</t>
-        </is>
-      </c>
-      <c r="B11" s="86" t="n">
-        <v>18.26</v>
-      </c>
-      <c r="C11" s="86" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="D11" s="86" t="n">
-        <v>8.01</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="85" t="inlineStr">
-        <is>
-          <t>24-09-2026</t>
-        </is>
-      </c>
-      <c r="B12" s="86" t="n">
-        <v>142.11</v>
-      </c>
-      <c r="C12" s="86" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="D12" s="86" t="n">
-        <v>81.48999999999999</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="85" t="inlineStr">
-        <is>
-          <t>25-09-2026</t>
-        </is>
-      </c>
-      <c r="B13" s="86" t="n">
-        <v>128.52</v>
-      </c>
-      <c r="C13" s="86" t="n">
-        <v>13</v>
-      </c>
-      <c r="D13" s="86" t="n">
-        <v>90.23999999999999</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="85" t="inlineStr">
-        <is>
-          <t>26-09-2026</t>
-        </is>
-      </c>
-      <c r="B14" s="86" t="n">
-        <v>98.81</v>
-      </c>
-      <c r="C14" s="86" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="D14" s="86" t="n">
-        <v>58.56</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="85" t="inlineStr">
-        <is>
-          <t>27-09-2026</t>
-        </is>
-      </c>
-      <c r="B15" s="86" t="n">
-        <v>82.17</v>
-      </c>
-      <c r="C15" s="86" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="D15" s="86" t="n">
-        <v>66.52</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="85" t="inlineStr">
-        <is>
-          <t>28-09-2026</t>
-        </is>
-      </c>
-      <c r="B16" s="86" t="n">
-        <v>109.52</v>
-      </c>
-      <c r="C16" s="86" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="D16" s="86" t="n">
-        <v>72.23</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="85" t="inlineStr">
-        <is>
-          <t>29-09-2026</t>
-        </is>
-      </c>
-      <c r="B17" s="86" t="n">
-        <v>120.97</v>
-      </c>
-      <c r="C17" s="86" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="D17" s="86" t="n">
-        <v>80.69</v>
+      <c r="F16" s="94" t="n">
+        <v>2021.28</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="85" t="inlineStr">
-        <is>
-          <t>30-09-2026</t>
-        </is>
-      </c>
-      <c r="B18" s="86" t="n">
-        <v>170.73</v>
-      </c>
-      <c r="C18" s="86" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="D18" s="86" t="n">
-        <v>106.17</v>
+      <c r="A18" s="83" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="85" t="inlineStr">
-        <is>
-          <t>01-10-2026</t>
-        </is>
-      </c>
-      <c r="B19" s="86" t="n">
-        <v>158.2</v>
-      </c>
-      <c r="C19" s="86" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="D19" s="86" t="n">
-        <v>111.39</v>
+      <c r="A19" s="95" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL (000027-01): 1.271,28 m³ en 207 horas.</t>
+        </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="85" t="inlineStr">
-        <is>
-          <t>02-10-2026 hasta 07:00</t>
-        </is>
-      </c>
-      <c r="B20" s="86" t="n">
-        <v>70.81</v>
-      </c>
-      <c r="C20" s="86" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="D20" s="86" t="n">
-        <v>50.28</v>
+      <c r="A20" s="95" t="inlineStr">
+        <is>
+          <t>Estanque Inferior (000027-02): 1.100,10 m³ en 207 horas.</t>
+        </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="87" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B21" s="88" t="n">
-        <v>1100.1</v>
-      </c>
-      <c r="C21" s="88" t="n">
-        <v>195.6</v>
-      </c>
-      <c r="D21" s="88" t="n">
-        <v>725.58</v>
+      <c r="A21" s="95" t="inlineStr">
+        <is>
+          <t>Etapa N°5 (000027-03): 195,60 m³ en 207 horas. Misma ventana de la relojería 5.174 → 5.369 m³.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="95" t="inlineStr">
+        <is>
+          <t>Etapa 1 al 4 (000027-04): 725,58 m³ en 206 horas. Falta la hora 14:00 del 24-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="95" t="inlineStr">
+        <is>
+          <t>Total: Estanque Inferior + Etapa N°5 + Etapa 1 al 4 = 2.021,28 m³.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E7"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+  <autoFilter ref="A5:F15"/>
+  <mergeCells count="8">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LFundo Zapallar&amp;R23-09 16:54 a 02-10 08:44</oddHeader>

</xml_diff>

<commit_message>
Add stacked daily bars for daytime and night on the Fundo window.
Night is 00:00 to 06:00 and daytime is from 06:00, for Matriz ESVAL, Estanque Inferior, Etapa 5 and Etapa 1 al 4.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -42,7 +42,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -115,8 +115,19 @@
       <color rgb="001F4E79"/>
       <sz val="13"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00475569"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -166,6 +177,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF4CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -253,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -496,6 +522,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -573,6 +613,522 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Matriz ESVAL</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Misma ventana'!B29</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E75B6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Misma ventana'!$A$30:$A$39</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Misma ventana'!$B$30:$B$39</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Misma ventana'!C29</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FFC000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Misma ventana'!$A$30:$A$39</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Misma ventana'!$C$30:$C$39</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Estanque Inferior</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Misma ventana'!D29</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E75B6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Misma ventana'!$A$30:$A$39</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Misma ventana'!$D$30:$D$39</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Misma ventana'!E29</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FFC000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Misma ventana'!$A$30:$A$39</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Misma ventana'!$E$30:$E$39</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Etapa N°5</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Misma ventana'!F29</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E75B6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Misma ventana'!$A$30:$A$39</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Misma ventana'!$F$30:$F$39</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Misma ventana'!G29</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FFC000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Misma ventana'!$A$30:$A$39</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Misma ventana'!$G$30:$G$39</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Etapa 1 al 4</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Misma ventana'!H29</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E75B6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Misma ventana'!$A$30:$A$39</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Misma ventana'!$H$30:$H$39</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Misma ventana'!I29</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FFC000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Misma ventana'!$A$30:$A$39</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Misma ventana'!$I$30:$I$39</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -755,6 +1311,124 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>57</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>57</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9334500" cy="5905500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1300,7 +1974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1648,28 +2322,433 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="83" t="inlineStr">
+        <is>
+          <t>Día y noche por punto</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="96" t="inlineStr">
+        <is>
+          <t>Azul = día, desde las 06:00. Amarillo = noche, de 00:00 a 06:00 (horas 00, 01, 02, 03, 04 y 05). El 23-09 entra desde las 17:00 y el 02-10 llega hasta las 08:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="89" t="inlineStr">
+        <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="B29" s="97" t="inlineStr">
+        <is>
+          <t>Matriz día</t>
+        </is>
+      </c>
+      <c r="C29" s="98" t="inlineStr">
+        <is>
+          <t>Matriz noche</t>
+        </is>
+      </c>
+      <c r="D29" s="97" t="inlineStr">
+        <is>
+          <t>Inferior día</t>
+        </is>
+      </c>
+      <c r="E29" s="98" t="inlineStr">
+        <is>
+          <t>Inferior noche</t>
+        </is>
+      </c>
+      <c r="F29" s="97" t="inlineStr">
+        <is>
+          <t>Etapa 5 día</t>
+        </is>
+      </c>
+      <c r="G29" s="98" t="inlineStr">
+        <is>
+          <t>Etapa 5 noche</t>
+        </is>
+      </c>
+      <c r="H29" s="97" t="inlineStr">
+        <is>
+          <t>Etapa 1-4 día</t>
+        </is>
+      </c>
+      <c r="I29" s="98" t="inlineStr">
+        <is>
+          <t>Etapa 1-4 noche</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="99" t="inlineStr">
+        <is>
+          <t>23-09-2026 desde 17:00</t>
+        </is>
+      </c>
+      <c r="B30" s="91" t="n">
+        <v>24.17</v>
+      </c>
+      <c r="C30" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="91" t="n">
+        <v>18.26</v>
+      </c>
+      <c r="E30" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="91" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G30" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="91" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="I30" s="100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="99" t="inlineStr">
+        <is>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="B31" s="91" t="n">
+        <v>117.95</v>
+      </c>
+      <c r="C31" s="100" t="n">
+        <v>43.81</v>
+      </c>
+      <c r="D31" s="91" t="n">
+        <v>105.13</v>
+      </c>
+      <c r="E31" s="100" t="n">
+        <v>36.98</v>
+      </c>
+      <c r="F31" s="91" t="n">
+        <v>19</v>
+      </c>
+      <c r="G31" s="100" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H31" s="91" t="n">
+        <v>59.53</v>
+      </c>
+      <c r="I31" s="100" t="n">
+        <v>21.96</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="99" t="inlineStr">
+        <is>
+          <t>25-09-2026</t>
+        </is>
+      </c>
+      <c r="B32" s="91" t="n">
+        <v>110.63</v>
+      </c>
+      <c r="C32" s="100" t="n">
+        <v>37.98</v>
+      </c>
+      <c r="D32" s="91" t="n">
+        <v>95.79000000000001</v>
+      </c>
+      <c r="E32" s="100" t="n">
+        <v>32.73</v>
+      </c>
+      <c r="F32" s="91" t="n">
+        <v>13</v>
+      </c>
+      <c r="G32" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="91" t="n">
+        <v>62.92</v>
+      </c>
+      <c r="I32" s="100" t="n">
+        <v>27.32</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="99" t="inlineStr">
+        <is>
+          <t>26-09-2026</t>
+        </is>
+      </c>
+      <c r="B33" s="91" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="C33" s="100" t="n">
+        <v>42.45</v>
+      </c>
+      <c r="D33" s="91" t="n">
+        <v>64.13</v>
+      </c>
+      <c r="E33" s="100" t="n">
+        <v>34.68</v>
+      </c>
+      <c r="F33" s="91" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G33" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="91" t="n">
+        <v>31.67</v>
+      </c>
+      <c r="I33" s="100" t="n">
+        <v>26.89</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="99" t="inlineStr">
+        <is>
+          <t>27-09-2026</t>
+        </is>
+      </c>
+      <c r="B34" s="91" t="n">
+        <v>48.49</v>
+      </c>
+      <c r="C34" s="100" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="D34" s="91" t="n">
+        <v>41.15</v>
+      </c>
+      <c r="E34" s="100" t="n">
+        <v>41.02</v>
+      </c>
+      <c r="F34" s="91" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G34" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="91" t="n">
+        <v>32.12</v>
+      </c>
+      <c r="I34" s="100" t="n">
+        <v>34.4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="99" t="inlineStr">
+        <is>
+          <t>28-09-2026</t>
+        </is>
+      </c>
+      <c r="B35" s="91" t="n">
+        <v>79.20999999999999</v>
+      </c>
+      <c r="C35" s="100" t="n">
+        <v>48.61</v>
+      </c>
+      <c r="D35" s="91" t="n">
+        <v>67.59</v>
+      </c>
+      <c r="E35" s="100" t="n">
+        <v>41.93</v>
+      </c>
+      <c r="F35" s="91" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="G35" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="91" t="n">
+        <v>38.64</v>
+      </c>
+      <c r="I35" s="100" t="n">
+        <v>33.59</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="99" t="inlineStr">
+        <is>
+          <t>29-09-2026</t>
+        </is>
+      </c>
+      <c r="B36" s="91" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="C36" s="100" t="n">
+        <v>44.21</v>
+      </c>
+      <c r="D36" s="91" t="n">
+        <v>84.98</v>
+      </c>
+      <c r="E36" s="100" t="n">
+        <v>35.99</v>
+      </c>
+      <c r="F36" s="91" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="G36" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="91" t="n">
+        <v>49.49</v>
+      </c>
+      <c r="I36" s="100" t="n">
+        <v>31.2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="99" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="B37" s="91" t="n">
+        <v>130.8</v>
+      </c>
+      <c r="C37" s="100" t="n">
+        <v>60.36</v>
+      </c>
+      <c r="D37" s="91" t="n">
+        <v>117.49</v>
+      </c>
+      <c r="E37" s="100" t="n">
+        <v>53.24</v>
+      </c>
+      <c r="F37" s="91" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="G37" s="100" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H37" s="91" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="I37" s="100" t="n">
+        <v>37.87</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="99" t="inlineStr">
+        <is>
+          <t>01-10-2026</t>
+        </is>
+      </c>
+      <c r="B38" s="91" t="n">
+        <v>149.55</v>
+      </c>
+      <c r="C38" s="100" t="n">
+        <v>45.08</v>
+      </c>
+      <c r="D38" s="91" t="n">
+        <v>120.74</v>
+      </c>
+      <c r="E38" s="100" t="n">
+        <v>37.46</v>
+      </c>
+      <c r="F38" s="91" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="G38" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="91" t="n">
+        <v>78.78</v>
+      </c>
+      <c r="I38" s="100" t="n">
+        <v>32.61</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="99" t="inlineStr">
+        <is>
+          <t>02-10-2026 hasta 07:00</t>
+        </is>
+      </c>
+      <c r="B39" s="91" t="n">
+        <v>20.19</v>
+      </c>
+      <c r="C39" s="100" t="n">
+        <v>57.19</v>
+      </c>
+      <c r="D39" s="91" t="n">
+        <v>19.82</v>
+      </c>
+      <c r="E39" s="100" t="n">
+        <v>50.99</v>
+      </c>
+      <c r="F39" s="91" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G39" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="91" t="n">
+        <v>10.42</v>
+      </c>
+      <c r="I39" s="100" t="n">
+        <v>39.86</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="101" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B40" s="94" t="n">
+        <v>844.99</v>
+      </c>
+      <c r="C40" s="94" t="n">
+        <v>426.29</v>
+      </c>
+      <c r="D40" s="94" t="n">
+        <v>735.08</v>
+      </c>
+      <c r="E40" s="94" t="n">
+        <v>365.02</v>
+      </c>
+      <c r="F40" s="94" t="n">
+        <v>187.3</v>
+      </c>
+      <c r="G40" s="94" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H40" s="94" t="n">
+        <v>439.88</v>
+      </c>
+      <c r="I40" s="94" t="n">
+        <v>285.7</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A5:F15"/>
-  <mergeCells count="8">
+  <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A27:I27"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A26:I26"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LFundo Zapallar&amp;R23-09 16:54 a 02-10 08:44</oddHeader>
-    <oddFooter>&amp;LApp WES, horas completas&amp;RPágina &amp;P de &amp;N</oddFooter>
+    <oddHeader>&amp;LFundo Zapallar&amp;RDía y noche 00:00 a 06:00</oddHeader>
+    <oddFooter>&amp;LAzul = día desde las 06:00    Amarillo = noche 00:00 a 06:00&amp;RPágina &amp;P de &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Label day and night on the bars and add the balance gaps.
The chart shows each segment in cubic metres. Matriz ESVAL is 13.5% above Estanque Inferior, and the tank is 16.3% above Etapa 5 plus Etapa 1 al 4.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -42,7 +42,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -125,6 +125,12 @@
       <b val="1"/>
       <color rgb="001F2937"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="14">
@@ -279,7 +285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -536,6 +542,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -614,7 +621,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -743,7 +749,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -872,7 +877,6 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1001,7 +1005,6 @@
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1407,7 +1410,7 @@
       <row>75</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9334500" cy="5905500"/>
+    <ext cx="9334500" cy="6096000"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -2322,6 +2325,20 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="102" t="inlineStr">
+        <is>
+          <t>Diferencia Matriz ESVAL y Estanque Inferior: 171,18 m³, 13,5 % de la Matriz (1.271,28 − 1.100,10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="102" t="inlineStr">
+        <is>
+          <t>Diferencia Estanque Inferior y Etapa N°5 + Etapa 1 al 4: 178,92 m³, 16,3 % del Inferior (1.100,10 − 921,18).</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" s="83" t="inlineStr">
         <is>
@@ -2726,7 +2743,8 @@
     </row>
   </sheetData>
   <autoFilter ref="A5:F15"/>
-  <mergeCells count="10">
+  <mergeCells count="12">
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
@@ -2737,6 +2755,7 @@
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add hourly profiles for the four days that break the daily pattern.
26, 29 and 30 September and 1 October are broken out hour by hour for Matriz ESVAL, Estanque Inferior, Etapa 5 and Etapa 1 al 4.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -9,29 +9,31 @@
   <sheets>
     <sheet name="Relojeria" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Misma ventana" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lecturas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Horario hoy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Historico mensual" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cierre de indice" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Hallazgos" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Horas interesantes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Resumen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lecturas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Horario hoy" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Historico mensual" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cierre de indice" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Hallazgos" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relojeria'!$A$4:$J$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Relojeria'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Misma ventana'!$A$5:$F$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Misma ventana'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resumen'!$A$5:$C$22</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Resumen'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lecturas'!$A$4:$C$22</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Lecturas'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Horario hoy'!$A$4:$E$19</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Horario hoy'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Historico mensual'!$A$4:$G$21</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Historico mensual'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Cierre de indice'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Hallazgos'!$A$4:$D$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Hallazgos'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Horas interesantes'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Resumen'!$A$5:$C$22</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Resumen'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Lecturas'!$A$4:$C$22</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Lecturas'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Horario hoy'!$A$4:$E$19</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Horario hoy'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Historico mensual'!$A$4:$G$21</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Historico mensual'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Cierre de indice'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Hallazgos'!$A$4:$D$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Hallazgos'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,7 +44,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,6 +133,12 @@
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="14">
@@ -285,7 +293,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -543,6 +551,26 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1133,6 +1161,966 @@
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>26-09</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!B9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F4E79"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$10:$A$33</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$B$10:$B$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!C9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="5B9BD5"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$10:$A$33</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$C$10:$C$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!D9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E67E22"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="E67E22"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="E67E22"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$10:$A$33</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$D$10:$D$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!E9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2E7D32"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$10:$A$33</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$E$10:$E$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>29-09</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!B38</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F4E79"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$39:$A$62</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$B$39:$B$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!C38</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="5B9BD5"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$39:$A$62</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$C$39:$C$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!D38</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E67E22"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="E67E22"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="E67E22"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$39:$A$62</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$D$39:$D$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!E38</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2E7D32"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$39:$A$62</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$E$39:$E$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>30-09</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!B67</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F4E79"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$68:$A$91</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$B$68:$B$91</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!C67</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="5B9BD5"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$68:$A$91</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$C$68:$C$91</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!D67</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E67E22"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="E67E22"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="E67E22"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$68:$A$91</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$D$68:$D$91</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!E67</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2E7D32"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$68:$A$91</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$E$68:$E$91</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>01-10</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!B96</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F4E79"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$97:$A$120</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$B$97:$B$120</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!C96</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="5B9BD5"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$97:$A$120</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$C$97:$C$120</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!D96</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E67E22"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="E67E22"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="E67E22"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$97:$A$120</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$D$97:$D$120</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Horas interesantes'!E96</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2E7D32"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Horas interesantes'!$A$97:$A$120</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Horas interesantes'!$E$97:$E$120</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
@@ -1424,6 +2412,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1432,6 +2423,124 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>66</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>95</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>119</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9334500" cy="5905500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -2774,6 +3883,2448 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F121"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="103" t="inlineStr">
+        <is>
+          <t>Doble clic por hora  ·  26-09, 29-09, 30-09 y 01-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="96" t="inlineStr">
+        <is>
+          <t>Noche marcada en amarillo: 00:00 a 06:00. Valores en m³ de cada hora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="104" t="inlineStr">
+        <is>
+          <t>26-09. El Inferior queda 35,8 % sobre las etapas. Etapa N°5 casi no corre (4,90 m³). El estanque carga a las 13:00 (14,82 m³) y a las 23:00 (15,66 m³) y las etapas no lo siguen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="104" t="inlineStr">
+        <is>
+          <t>29-09. Las etapas superan al Inferior en 11,4 %. Etapa N°5 suma 43,0 m³ entre las 18:00 y las 23:00, con el estanque en cero a las 20:00 y a las 23:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="104" t="inlineStr">
+        <is>
+          <t>30-09. Día de más volumen. A las 16:00 se mueven juntos: Matriz 18,23, Inferior 17,06 y Etapa N°5 16,10. De noche Etapa N°5 marca 1,30 m³ cada hora, de 00:00 a 05:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="104" t="inlineStr">
+        <is>
+          <t>01-10. Mayor brecha Matriz–Inferior (18,7 %). Se concentra a las 16:00 (Matriz 7,29 contra Inferior 0,51) y a las 17:00 (21,80 contra 14,17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="103" t="inlineStr">
+        <is>
+          <t>26-09  ·  el Inferior queda 35,8 % sobre las etapas</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="105" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="B9" s="105" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL</t>
+        </is>
+      </c>
+      <c r="C9" s="105" t="inlineStr">
+        <is>
+          <t>Estanque Inferior</t>
+        </is>
+      </c>
+      <c r="D9" s="105" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="E9" s="105" t="inlineStr">
+        <is>
+          <t>Etapa 1 al 4</t>
+        </is>
+      </c>
+      <c r="F9" s="105" t="inlineStr">
+        <is>
+          <t>Etapa 5 + 1 al 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="106" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="B10" s="107" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="C10" s="107" t="n">
+        <v>8.44</v>
+      </c>
+      <c r="D10" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="107" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="F10" s="107" t="n">
+        <v>4.23</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="106" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="B11" s="107" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="C11" s="107" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="D11" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="107" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F11" s="107" t="n">
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="106" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="B12" s="107" t="n">
+        <v>9</v>
+      </c>
+      <c r="C12" s="107" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D12" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="107" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="F12" s="107" t="n">
+        <v>11.28</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="106" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="B13" s="107" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="C13" s="107" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="D13" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="107" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="F13" s="107" t="n">
+        <v>5.38</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="106" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="B14" s="107" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C14" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="107" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F14" s="107" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="106" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="B15" s="107" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C15" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="107" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F15" s="107" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="108" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="B16" s="109" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="C16" s="109" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="D16" s="109" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E16" s="109" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="F16" s="109" t="n">
+        <v>8.029999999999999</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="108" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B17" s="109" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="C17" s="109" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="D17" s="109" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E17" s="109" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="F17" s="109" t="n">
+        <v>2.13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="108" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="B18" s="109" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="C18" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="109" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F18" s="109" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="108" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B19" s="109" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="C19" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="109" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F19" s="109" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="108" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B20" s="109" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C20" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="109" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F20" s="109" t="n">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="108" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B21" s="109" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="C21" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="109" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E21" s="109" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="F21" s="109" t="n">
+        <v>3.03</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="108" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B22" s="109" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C22" s="109" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="D22" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="109" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="F22" s="109" t="n">
+        <v>3.21</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="108" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B23" s="109" t="n">
+        <v>15.88</v>
+      </c>
+      <c r="C23" s="109" t="n">
+        <v>14.82</v>
+      </c>
+      <c r="D23" s="109" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E23" s="109" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="F23" s="109" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="108" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B24" s="109" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="C24" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="109" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E24" s="109" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F24" s="109" t="n">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="108" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="B25" s="109" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="C25" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="109" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E25" s="109" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F25" s="109" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="B26" s="109" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C26" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="109" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F26" s="109" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="108" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B27" s="109" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="C27" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="109" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F27" s="109" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="108" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B28" s="109" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="C28" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="109" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F28" s="109" t="n">
+        <v>1.18</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="108" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B29" s="109" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="C29" s="109" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="D29" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="109" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F29" s="109" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="108" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="B30" s="109" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="C30" s="109" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="D30" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="109" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="F30" s="109" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="108" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="B31" s="109" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="C31" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="109" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="F31" s="109" t="n">
+        <v>4.29</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="108" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B32" s="109" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="C32" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="109" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F32" s="109" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="108" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B33" s="109" t="n">
+        <v>14.63</v>
+      </c>
+      <c r="C33" s="109" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="D33" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="109" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="F33" s="109" t="n">
+        <v>4.34</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="101" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B34" s="110" t="n">
+        <v>112.95</v>
+      </c>
+      <c r="C34" s="110" t="n">
+        <v>98.81</v>
+      </c>
+      <c r="D34" s="110" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E34" s="110" t="n">
+        <v>58.56</v>
+      </c>
+      <c r="F34" s="110" t="n">
+        <v>63.46</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="103" t="inlineStr">
+        <is>
+          <t>29-09  ·  las etapas superan al Inferior en 11,4 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="105" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="B38" s="105" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL</t>
+        </is>
+      </c>
+      <c r="C38" s="105" t="inlineStr">
+        <is>
+          <t>Estanque Inferior</t>
+        </is>
+      </c>
+      <c r="D38" s="105" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="E38" s="105" t="inlineStr">
+        <is>
+          <t>Etapa 1 al 4</t>
+        </is>
+      </c>
+      <c r="F38" s="105" t="inlineStr">
+        <is>
+          <t>Etapa 5 + 1 al 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="106" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="B39" s="107" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="C39" s="107" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="D39" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="107" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="F39" s="107" t="n">
+        <v>3.92</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="106" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="B40" s="107" t="n">
+        <v>14.11</v>
+      </c>
+      <c r="C40" s="107" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="D40" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="107" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="F40" s="107" t="n">
+        <v>3.54</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="106" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="B41" s="107" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="C41" s="107" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="D41" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="107" t="n">
+        <v>13.08</v>
+      </c>
+      <c r="F41" s="107" t="n">
+        <v>13.08</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="106" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="B42" s="107" t="n">
+        <v>17.53</v>
+      </c>
+      <c r="C42" s="107" t="n">
+        <v>15.14</v>
+      </c>
+      <c r="D42" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="107" t="n">
+        <v>5.74</v>
+      </c>
+      <c r="F42" s="107" t="n">
+        <v>5.74</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="106" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="B43" s="107" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="C43" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="107" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F43" s="107" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="106" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="B44" s="107" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="C44" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="107" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F44" s="107" t="n">
+        <v>1.43</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="108" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="B45" s="109" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="C45" s="109" t="n">
+        <v>6</v>
+      </c>
+      <c r="D45" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="109" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="F45" s="109" t="n">
+        <v>5.82</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="108" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B46" s="109" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="C46" s="109" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="D46" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="109" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="F46" s="109" t="n">
+        <v>3.82</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="108" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="B47" s="109" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C47" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="109" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="F47" s="109" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="108" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B48" s="109" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="C48" s="109" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D48" s="109" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E48" s="109" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="F48" s="109" t="n">
+        <v>4.64</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="108" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B49" s="109" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="C49" s="109" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="D49" s="109" t="n">
+        <v>5</v>
+      </c>
+      <c r="E49" s="109" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F49" s="109" t="n">
+        <v>6.92</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="108" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B50" s="109" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="C50" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="109" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="109" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="F50" s="109" t="n">
+        <v>2.71</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="108" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B51" s="109" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C51" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="109" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E51" s="109" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="F51" s="109" t="n">
+        <v>2.87</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="108" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B52" s="109" t="n">
+        <v>14</v>
+      </c>
+      <c r="C52" s="109" t="n">
+        <v>14.07</v>
+      </c>
+      <c r="D52" s="109" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="109" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="F52" s="109" t="n">
+        <v>4.09</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="108" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B53" s="109" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C53" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="109" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E53" s="109" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F53" s="109" t="n">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="108" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="B54" s="109" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="C54" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="109" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E54" s="109" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F54" s="109" t="n">
+        <v>3.77</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="B55" s="109" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C55" s="109" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="D55" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="109" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="F55" s="109" t="n">
+        <v>4.17</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="108" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B56" s="109" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="C56" s="109" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="D56" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="109" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F56" s="109" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="108" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B57" s="109" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="C57" s="109" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D57" s="109" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E57" s="109" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F57" s="109" t="n">
+        <v>8.25</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="108" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B58" s="109" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="C58" s="109" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="D58" s="109" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="E58" s="109" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="F58" s="109" t="n">
+        <v>8.640000000000001</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="108" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="B59" s="109" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C59" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="109" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E59" s="109" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="F59" s="109" t="n">
+        <v>9.06</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="108" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="B60" s="109" t="n">
+        <v>7.61</v>
+      </c>
+      <c r="C60" s="109" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="D60" s="109" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E60" s="109" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="F60" s="109" t="n">
+        <v>12.96</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="108" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B61" s="109" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="C61" s="109" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="D61" s="109" t="n">
+        <v>7</v>
+      </c>
+      <c r="E61" s="109" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="F61" s="109" t="n">
+        <v>11.74</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="108" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B62" s="109" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C62" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" s="109" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E62" s="109" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="F62" s="109" t="n">
+        <v>10.14</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="101" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B63" s="110" t="n">
+        <v>137.71</v>
+      </c>
+      <c r="C63" s="110" t="n">
+        <v>120.97</v>
+      </c>
+      <c r="D63" s="110" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="E63" s="110" t="n">
+        <v>80.69</v>
+      </c>
+      <c r="F63" s="110" t="n">
+        <v>134.79</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="103" t="inlineStr">
+        <is>
+          <t>30-09  ·  mayor volumen y pico de Etapa N°5 a las 16:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="105" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="B67" s="105" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL</t>
+        </is>
+      </c>
+      <c r="C67" s="105" t="inlineStr">
+        <is>
+          <t>Estanque Inferior</t>
+        </is>
+      </c>
+      <c r="D67" s="105" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="E67" s="105" t="inlineStr">
+        <is>
+          <t>Etapa 1 al 4</t>
+        </is>
+      </c>
+      <c r="F67" s="105" t="inlineStr">
+        <is>
+          <t>Etapa 5 + 1 al 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="106" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="B68" s="107" t="n">
+        <v>21.27</v>
+      </c>
+      <c r="C68" s="107" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="D68" s="107" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E68" s="107" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="F68" s="107" t="n">
+        <v>6.62</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="106" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="B69" s="107" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="C69" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="107" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E69" s="107" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="F69" s="107" t="n">
+        <v>4.44</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="106" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="B70" s="107" t="n">
+        <v>9.26</v>
+      </c>
+      <c r="C70" s="107" t="n">
+        <v>9.48</v>
+      </c>
+      <c r="D70" s="107" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E70" s="107" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="F70" s="107" t="n">
+        <v>13.58</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="106" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="B71" s="107" t="n">
+        <v>17.94</v>
+      </c>
+      <c r="C71" s="107" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="D71" s="107" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E71" s="107" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="F71" s="107" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="106" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="B72" s="107" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="C72" s="107" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="D72" s="107" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E72" s="107" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="F72" s="107" t="n">
+        <v>7.86</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="106" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="B73" s="107" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="C73" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="107" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E73" s="107" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="F73" s="107" t="n">
+        <v>4.97</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="108" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="B74" s="109" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="C74" s="109" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="D74" s="109" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E74" s="109" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="F74" s="109" t="n">
+        <v>8.050000000000001</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="108" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B75" s="109" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="C75" s="109" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="D75" s="109" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E75" s="109" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="F75" s="109" t="n">
+        <v>3.68</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="108" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="B76" s="109" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C76" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="109" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E76" s="109" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="F76" s="109" t="n">
+        <v>2.91</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="108" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B77" s="109" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="C77" s="109" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="D77" s="109" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E77" s="109" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="F77" s="109" t="n">
+        <v>5.67</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="108" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B78" s="109" t="n">
+        <v>15.56</v>
+      </c>
+      <c r="C78" s="109" t="n">
+        <v>13.18</v>
+      </c>
+      <c r="D78" s="109" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E78" s="109" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F78" s="109" t="n">
+        <v>7.41</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="108" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B79" s="109" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="C79" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="109" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E79" s="109" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="F79" s="109" t="n">
+        <v>5.19</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="108" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B80" s="109" t="n">
+        <v>8.44</v>
+      </c>
+      <c r="C80" s="109" t="n">
+        <v>8.56</v>
+      </c>
+      <c r="D80" s="109" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E80" s="109" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="F80" s="109" t="n">
+        <v>9.050000000000001</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="108" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B81" s="109" t="n">
+        <v>16.93</v>
+      </c>
+      <c r="C81" s="109" t="n">
+        <v>15.17</v>
+      </c>
+      <c r="D81" s="109" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E81" s="109" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="F81" s="109" t="n">
+        <v>7.71</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="108" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B82" s="109" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="C82" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="109" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E82" s="109" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="F82" s="109" t="n">
+        <v>6.62</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="108" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="B83" s="109" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="C83" s="109" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="D83" s="109" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E83" s="109" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F83" s="109" t="n">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="B84" s="109" t="n">
+        <v>18.23</v>
+      </c>
+      <c r="C84" s="109" t="n">
+        <v>17.06</v>
+      </c>
+      <c r="D84" s="109" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="E84" s="109" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="F84" s="109" t="n">
+        <v>20.56</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="108" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B85" s="109" t="n">
+        <v>16.38</v>
+      </c>
+      <c r="C85" s="109" t="n">
+        <v>14.86</v>
+      </c>
+      <c r="D85" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="109" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F85" s="109" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="108" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B86" s="109" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="C86" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="109" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E86" s="109" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="F86" s="109" t="n">
+        <v>10.27</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="108" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B87" s="109" t="n">
+        <v>9.529999999999999</v>
+      </c>
+      <c r="C87" s="109" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="D87" s="109" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E87" s="109" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F87" s="109" t="n">
+        <v>5.03</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="108" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="B88" s="109" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="C88" s="109" t="n">
+        <v>3</v>
+      </c>
+      <c r="D88" s="109" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E88" s="109" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="F88" s="109" t="n">
+        <v>2.57</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="108" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="B89" s="109" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="C89" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="109" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="F89" s="109" t="n">
+        <v>3.84</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="108" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B90" s="109" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C90" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" s="109" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F90" s="109" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="108" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B91" s="109" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="C91" s="109" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D91" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="109" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="F91" s="109" t="n">
+        <v>3.03</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="101" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B92" s="110" t="n">
+        <v>191.16</v>
+      </c>
+      <c r="C92" s="110" t="n">
+        <v>170.73</v>
+      </c>
+      <c r="D92" s="110" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="E92" s="110" t="n">
+        <v>106.17</v>
+      </c>
+      <c r="F92" s="110" t="n">
+        <v>158.77</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="103" t="inlineStr">
+        <is>
+          <t>01-10  ·  mayor brecha Matriz–Inferior, 18,7 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="105" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="B96" s="105" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL</t>
+        </is>
+      </c>
+      <c r="C96" s="105" t="inlineStr">
+        <is>
+          <t>Estanque Inferior</t>
+        </is>
+      </c>
+      <c r="D96" s="105" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="E96" s="105" t="inlineStr">
+        <is>
+          <t>Etapa 1 al 4</t>
+        </is>
+      </c>
+      <c r="F96" s="105" t="inlineStr">
+        <is>
+          <t>Etapa 5 + 1 al 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="106" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="B97" s="107" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="C97" s="107" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="D97" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="107" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="F97" s="107" t="n">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="106" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="B98" s="107" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="C98" s="107" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="D98" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" s="107" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F98" s="107" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="106" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="B99" s="107" t="n">
+        <v>19.86</v>
+      </c>
+      <c r="C99" s="107" t="n">
+        <v>18.11</v>
+      </c>
+      <c r="D99" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="107" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="F99" s="107" t="n">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="106" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="B100" s="107" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="C100" s="107" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="D100" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="107" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="F100" s="107" t="n">
+        <v>5.48</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="106" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="B101" s="107" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="C101" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D101" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="107" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F101" s="107" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="106" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="B102" s="107" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="C102" s="107" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="D102" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="107" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="F102" s="107" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="108" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="B103" s="109" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="C103" s="109" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="D103" s="109" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E103" s="109" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="F103" s="109" t="n">
+        <v>9.33</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="108" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B104" s="109" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C104" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D104" s="109" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="109" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="F104" s="109" t="n">
+        <v>5.32</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="108" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="B105" s="109" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="C105" s="109" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="D105" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="109" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="F105" s="109" t="n">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="108" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B106" s="109" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="C106" s="109" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="D106" s="109" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E106" s="109" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F106" s="109" t="n">
+        <v>3.85</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="108" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B107" s="109" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="C107" s="109" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="D107" s="109" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E107" s="109" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="F107" s="109" t="n">
+        <v>5.41</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="108" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B108" s="109" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="C108" s="109" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="D108" s="109" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E108" s="109" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="F108" s="109" t="n">
+        <v>6.87</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="108" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B109" s="109" t="n">
+        <v>19.06</v>
+      </c>
+      <c r="C109" s="109" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="D109" s="109" t="n">
+        <v>3</v>
+      </c>
+      <c r="E109" s="109" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F109" s="109" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="108" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B110" s="109" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="C110" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" s="109" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E110" s="109" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="F110" s="109" t="n">
+        <v>5.54</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="108" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B111" s="109" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="C111" s="109" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="D111" s="109" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E111" s="109" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="F111" s="109" t="n">
+        <v>6.34</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="108" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="B112" s="109" t="n">
+        <v>21.67</v>
+      </c>
+      <c r="C112" s="109" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="D112" s="109" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E112" s="109" t="n">
+        <v>5.97</v>
+      </c>
+      <c r="F112" s="109" t="n">
+        <v>9.07</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="108" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="B113" s="109" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="C113" s="109" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="D113" s="109" t="n">
+        <v>2</v>
+      </c>
+      <c r="E113" s="109" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="F113" s="109" t="n">
+        <v>9.58</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="108" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B114" s="109" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="C114" s="109" t="n">
+        <v>14.17</v>
+      </c>
+      <c r="D114" s="109" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E114" s="109" t="n">
+        <v>8.94</v>
+      </c>
+      <c r="F114" s="109" t="n">
+        <v>11.54</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="108" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B115" s="109" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="C115" s="109" t="n">
+        <v>13.22</v>
+      </c>
+      <c r="D115" s="109" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E115" s="109" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="F115" s="109" t="n">
+        <v>5.14</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="108" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B116" s="109" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="C116" s="109" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="D116" s="109" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E116" s="109" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="F116" s="109" t="n">
+        <v>2.07</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="108" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="B117" s="109" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="C117" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" s="109" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E117" s="109" t="n">
+        <v>3</v>
+      </c>
+      <c r="F117" s="109" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="108" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="B118" s="109" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="C118" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" s="109" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E118" s="109" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="F118" s="109" t="n">
+        <v>4.03</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="108" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B119" s="109" t="n">
+        <v>12.68</v>
+      </c>
+      <c r="C119" s="109" t="n">
+        <v>12.67</v>
+      </c>
+      <c r="D119" s="109" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E119" s="109" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F119" s="109" t="n">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="108" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B120" s="109" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="C120" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D120" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E120" s="109" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="F120" s="109" t="n">
+        <v>2.73</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="101" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B121" s="110" t="n">
+        <v>194.63</v>
+      </c>
+      <c r="C121" s="110" t="n">
+        <v>158.2</v>
+      </c>
+      <c r="D121" s="110" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="E121" s="110" t="n">
+        <v>111.39</v>
+      </c>
+      <c r="F121" s="110" t="n">
+        <v>133.59</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A95:F95"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;LFundo Zapallar&amp;RHoras de los días interesantes</oddHeader>
+    <oddFooter>&amp;LNoche 00:00 a 06:00 en amarillo&amp;RPágina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001F4788"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -3348,7 +6899,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00548235"/>
@@ -3715,7 +7266,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
@@ -4091,7 +7642,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C65911"/>
@@ -4635,7 +8186,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -5004,7 +8555,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>

</xml_diff>

<commit_message>
Treat the meter gaps as water left stored in the tanks.
Matriz ESVAL fills the lower tank and its outlet fills the upper tank. Etapa 5 and Etapa 1 al 4 leave the upper tank, so the balance is stored volume.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -9,31 +9,34 @@
   <sheets>
     <sheet name="Relojeria" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Misma ventana" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Horas interesantes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Resumen" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lecturas" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Horario hoy" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Historico mensual" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Cierre de indice" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Hallazgos" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Almacenado" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Horas interesantes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Resumen" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Lecturas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Horario hoy" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Historico mensual" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Cierre de indice" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Hallazgos" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relojeria'!$A$4:$J$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Relojeria'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Misma ventana'!$A$5:$F$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Misma ventana'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Horas interesantes'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Resumen'!$A$5:$C$22</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Resumen'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Lecturas'!$A$4:$C$22</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Lecturas'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Horario hoy'!$A$4:$E$19</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Horario hoy'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Historico mensual'!$A$4:$G$21</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Historico mensual'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Cierre de indice'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Hallazgos'!$A$4:$D$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Hallazgos'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Almacenado'!$A$4:$F$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Almacenado'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Horas interesantes'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Resumen'!$A$5:$C$22</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Resumen'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Lecturas'!$A$4:$C$22</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Lecturas'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Horario hoy'!$A$4:$E$19</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Horario hoy'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Historico mensual'!$A$4:$G$21</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Historico mensual'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Cierre de indice'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Hallazgos'!$A$4:$D$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Hallazgos'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,7 +47,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -140,8 +143,19 @@
       <color rgb="001F4E79"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="009A3412"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -206,6 +220,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF4CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEDD5"/>
       </patternFill>
     </fill>
   </fills>
@@ -293,7 +312,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -571,6 +590,14 @@
     <xf numFmtId="4" fontId="4" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="18" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -761,6 +788,127 @@
             </rich>
           </tx>
         </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>m³ por mes</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Historico mensual'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Historico mensual'!$A$5:$A$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Historico mensual'!$B$5:$B$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Historico mensual'!D4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Historico mensual'!$A$5:$A$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Historico mensual'!$D$5:$D$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1172,6 +1320,133 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>m³ que quedan en cada estanque</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Almacenado'!H4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F4E79"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Almacenado'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Almacenado'!$H$5:$H$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Almacenado'!I4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="5B9BD5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Almacenado'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Almacenado'!$I$5:$I$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>m³</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>26-09</a:t>
             </a:r>
           </a:p>
@@ -1399,9 +1674,8 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1639,9 +1913,8 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1879,9 +2152,8 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -2119,127 +2391,6 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>m³ por mes</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Historico mensual'!B4</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Historico mensual'!$A$5:$A$21</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Historico mensual'!$B$5:$B$21</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Historico mensual'!D4</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Historico mensual'!$A$5:$A$21</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Historico mensual'!$D$5:$D$21</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>m³</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="b"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -2426,6 +2577,33 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>7</col>
       <colOff>0</colOff>
       <row>8</row>
@@ -2533,6 +2711,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2540,7 +2721,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -3080,6 +3261,225 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C00000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Hallazgos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Ordenados para revisar en terreno. El detalle numérico está en las otras hojas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Punto</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Situación</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Qué se encontró</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="53" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>Validado</t>
+        </is>
+      </c>
+      <c r="D5" s="74" t="inlineStr">
+        <is>
+          <t>La foto del viernes 02-10 es el mismo Sensus del informe (serie SEN01 2370 9030). La lectura inicial es 5.174 m³ a las 16:54 del 23-09. El viernes a las 08:44 marca 5.369 m³.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="62" customHeight="1">
+      <c r="A6" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="55" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>Relojería vs app</t>
+        </is>
+      </c>
+      <c r="D6" s="75" t="inlineStr">
+        <is>
+          <t>Del 23-09 17:00 al 02-10 08:00 (horas de las fotos fuera de la suma) la relojería avanza 195,0 m³ y la app suma 195,6 m³. Error 0,3 % (1 − 195,0/195,6). 207 horas. Desde el 28-09 08:57 (5.225 m³) hasta el viernes la relojería avanza 144 m³ y la app 148,0 m³ (error 2,7 %).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="62" customHeight="1">
+      <c r="A7" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="43" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Marzo 2026 no usable</t>
+        </is>
+      </c>
+      <c r="D7" s="57" t="inlineStr">
+        <is>
+          <t>En marzo 2026 Etapa N°5 marca 17.873,4 m³ y la Matriz 1.987,0 m³. Con ese mes, el histórico de WES (32.269,0 m³) supera toda la vida del medidor. Mayo 2026 también queda parejo con la Matriz (Etapa 5 un poco por encima) y conviene mirarlo aparte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="62" customHeight="1">
+      <c r="A8" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="53" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Medidor identificado</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>La foto de hoy es el mismo Itron Flostar S del informe, en Los Portones 378. El 23-09-2026 a las 17:05 marcaba 384.148,9 m³. Hoy a las 13:22 marca 385.430,8 m³. Relojería 1.281,9 m³ contra app 1.309,6 m³: error 2,1 %, del mismo orden que el 3,7 % del 23–28/09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="62" customHeight="1">
+      <c r="A9" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Telemetría detenida</t>
+        </is>
+      </c>
+      <c r="D9" s="57" t="inlineStr">
+        <is>
+          <t>Última trama 021026 14:14. La foto es de las 13:22, con el punto ya mudo. A las 14:25 llevaba 12 min sin muestras. Etapa N°5, Estanque Inferior y Etapa 1 al 4 tenían trama dentro de los últimos 10 minutos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="62" customHeight="1">
+      <c r="A10" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="55" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>m³ y L/min no cierran</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>No hubo muestras suficientes para recalcular el desfase en esta consulta. Con una sola foto no se sabe cuál de los dos canales está bien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="62" customHeight="1">
+      <c r="A11" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>Etapa N°5</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>Hora de la foto</t>
+        </is>
+      </c>
+      <c r="D11" s="52" t="inlineStr">
+        <is>
+          <t>La validación se pidió con la foto 1 de las 05:00. La hora impresa en esa foto es 08:44. A las 05:00 Etapa N°5 marcaba 0,00 m³, igual que desde la medianoche. A las 08:00 el balde horario es 0,10 m³.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="58" t="inlineStr">
+        <is>
+          <t>Siguiente paso para cerrar la Matriz: segunda lectura del mismo Flostar y revisión en terreno de por qué no volvió a transmitir después de las 13:14.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:D11"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;RPágina &amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3434,17 +3834,17 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="102" t="inlineStr">
-        <is>
-          <t>Diferencia Matriz ESVAL y Estanque Inferior: 171,18 m³, 13,5 % de la Matriz (1.271,28 − 1.100,10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="102" t="inlineStr">
-        <is>
-          <t>Diferencia Estanque Inferior y Etapa N°5 + Etapa 1 al 4: 178,92 m³, 16,3 % del Inferior (1.100,10 − 921,18).</t>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="111" t="inlineStr">
+        <is>
+          <t>Estanque Inferior. Matriz ESVAL lo llena y el medidor del estanque es su salida. Quedan almacenados 171,18 m³ (1.271,28 − 1.100,10), un 13,5 % de la Matriz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="111" t="inlineStr">
+        <is>
+          <t>Estanque Superior. Lo llena la salida del Inferior. Etapa N°5 y Etapa 1 al 4 son su salida. Quedan almacenados 178,92 m³ (1.100,10 − 921,18), un 16,3 % de la salida del Inferior.</t>
         </is>
       </c>
     </row>
@@ -3886,6 +4286,422 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>Agua que queda almacenada en los estanques</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="112" t="inlineStr">
+        <is>
+          <t>Matriz ESVAL llena el estanque inferior. La salida del inferior llena el estanque superior. Etapa N°5 y Etapa 1 al 4 son la salida del superior. Lo que entra y no sale queda almacenado. Un valor negativo es agua que el estanque entregó de lo que ya tenía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="89" t="inlineStr">
+        <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="B4" s="89" t="inlineStr">
+        <is>
+          <t>Entra al inferior
+Matriz ESVAL</t>
+        </is>
+      </c>
+      <c r="C4" s="89" t="inlineStr">
+        <is>
+          <t>Sale del inferior</t>
+        </is>
+      </c>
+      <c r="D4" s="89" t="inlineStr">
+        <is>
+          <t>Queda en el inferior</t>
+        </is>
+      </c>
+      <c r="E4" s="89" t="inlineStr">
+        <is>
+          <t>Sale del superior
+Etapa 5 + 1 al 4</t>
+        </is>
+      </c>
+      <c r="F4" s="89" t="inlineStr">
+        <is>
+          <t>Queda en el superior</t>
+        </is>
+      </c>
+      <c r="H4" s="84" t="inlineStr">
+        <is>
+          <t>Queda en el inferior</t>
+        </is>
+      </c>
+      <c r="I4" s="84" t="inlineStr">
+        <is>
+          <t>Queda en el superior</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="90" t="inlineStr">
+        <is>
+          <t>23-09 desde 17:00</t>
+        </is>
+      </c>
+      <c r="B5" s="91" t="n">
+        <v>24.17</v>
+      </c>
+      <c r="C5" s="91" t="n">
+        <v>18.26</v>
+      </c>
+      <c r="D5" s="91" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="E5" s="91" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="F5" s="91" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="H5" s="113" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="I5" s="113" t="n">
+        <v>9.35</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="90" t="inlineStr">
+        <is>
+          <t>24-09</t>
+        </is>
+      </c>
+      <c r="B6" s="91" t="n">
+        <v>161.76</v>
+      </c>
+      <c r="C6" s="91" t="n">
+        <v>142.11</v>
+      </c>
+      <c r="D6" s="91" t="n">
+        <v>19.65</v>
+      </c>
+      <c r="E6" s="91" t="n">
+        <v>100.99</v>
+      </c>
+      <c r="F6" s="91" t="n">
+        <v>41.12</v>
+      </c>
+      <c r="H6" s="113" t="n">
+        <v>19.65</v>
+      </c>
+      <c r="I6" s="113" t="n">
+        <v>41.12</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="90" t="inlineStr">
+        <is>
+          <t>25-09</t>
+        </is>
+      </c>
+      <c r="B7" s="91" t="n">
+        <v>148.61</v>
+      </c>
+      <c r="C7" s="91" t="n">
+        <v>128.52</v>
+      </c>
+      <c r="D7" s="91" t="n">
+        <v>20.09</v>
+      </c>
+      <c r="E7" s="91" t="n">
+        <v>103.24</v>
+      </c>
+      <c r="F7" s="91" t="n">
+        <v>25.28</v>
+      </c>
+      <c r="H7" s="113" t="n">
+        <v>20.09</v>
+      </c>
+      <c r="I7" s="113" t="n">
+        <v>25.28</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="90" t="inlineStr">
+        <is>
+          <t>26-09</t>
+        </is>
+      </c>
+      <c r="B8" s="91" t="n">
+        <v>112.95</v>
+      </c>
+      <c r="C8" s="91" t="n">
+        <v>98.81</v>
+      </c>
+      <c r="D8" s="91" t="n">
+        <v>14.14</v>
+      </c>
+      <c r="E8" s="91" t="n">
+        <v>63.46</v>
+      </c>
+      <c r="F8" s="91" t="n">
+        <v>35.35</v>
+      </c>
+      <c r="H8" s="113" t="n">
+        <v>14.14</v>
+      </c>
+      <c r="I8" s="113" t="n">
+        <v>35.35</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="90" t="inlineStr">
+        <is>
+          <t>27-09</t>
+        </is>
+      </c>
+      <c r="B9" s="91" t="n">
+        <v>95.09</v>
+      </c>
+      <c r="C9" s="91" t="n">
+        <v>82.17</v>
+      </c>
+      <c r="D9" s="91" t="n">
+        <v>12.92</v>
+      </c>
+      <c r="E9" s="91" t="n">
+        <v>71.42</v>
+      </c>
+      <c r="F9" s="91" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="H9" s="113" t="n">
+        <v>12.92</v>
+      </c>
+      <c r="I9" s="113" t="n">
+        <v>10.75</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="90" t="inlineStr">
+        <is>
+          <t>28-09</t>
+        </is>
+      </c>
+      <c r="B10" s="91" t="n">
+        <v>127.82</v>
+      </c>
+      <c r="C10" s="91" t="n">
+        <v>109.52</v>
+      </c>
+      <c r="D10" s="91" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="E10" s="91" t="n">
+        <v>91.53</v>
+      </c>
+      <c r="F10" s="91" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="H10" s="113" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="I10" s="113" t="n">
+        <v>17.99</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="90" t="inlineStr">
+        <is>
+          <t>29-09</t>
+        </is>
+      </c>
+      <c r="B11" s="91" t="n">
+        <v>137.71</v>
+      </c>
+      <c r="C11" s="91" t="n">
+        <v>120.97</v>
+      </c>
+      <c r="D11" s="91" t="n">
+        <v>16.74</v>
+      </c>
+      <c r="E11" s="91" t="n">
+        <v>134.79</v>
+      </c>
+      <c r="F11" s="114" t="n">
+        <v>-13.82</v>
+      </c>
+      <c r="H11" s="113" t="n">
+        <v>16.74</v>
+      </c>
+      <c r="I11" s="113" t="n">
+        <v>-13.82</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="90" t="inlineStr">
+        <is>
+          <t>30-09</t>
+        </is>
+      </c>
+      <c r="B12" s="91" t="n">
+        <v>191.16</v>
+      </c>
+      <c r="C12" s="91" t="n">
+        <v>170.73</v>
+      </c>
+      <c r="D12" s="91" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="E12" s="91" t="n">
+        <v>158.77</v>
+      </c>
+      <c r="F12" s="91" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="H12" s="113" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="I12" s="113" t="n">
+        <v>11.96</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="90" t="inlineStr">
+        <is>
+          <t>01-10</t>
+        </is>
+      </c>
+      <c r="B13" s="91" t="n">
+        <v>194.63</v>
+      </c>
+      <c r="C13" s="91" t="n">
+        <v>158.2</v>
+      </c>
+      <c r="D13" s="91" t="n">
+        <v>36.43</v>
+      </c>
+      <c r="E13" s="91" t="n">
+        <v>133.59</v>
+      </c>
+      <c r="F13" s="91" t="n">
+        <v>24.61</v>
+      </c>
+      <c r="H13" s="113" t="n">
+        <v>36.43</v>
+      </c>
+      <c r="I13" s="113" t="n">
+        <v>24.61</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="90" t="inlineStr">
+        <is>
+          <t>02-10 hasta 07:00</t>
+        </is>
+      </c>
+      <c r="B14" s="91" t="n">
+        <v>77.38</v>
+      </c>
+      <c r="C14" s="91" t="n">
+        <v>70.81</v>
+      </c>
+      <c r="D14" s="91" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="E14" s="91" t="n">
+        <v>54.48</v>
+      </c>
+      <c r="F14" s="91" t="n">
+        <v>16.33</v>
+      </c>
+      <c r="H14" s="113" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="I14" s="113" t="n">
+        <v>16.33</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="101" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B15" s="94" t="n">
+        <v>1271.28</v>
+      </c>
+      <c r="C15" s="94" t="n">
+        <v>1100.1</v>
+      </c>
+      <c r="D15" s="94" t="n">
+        <v>171.18</v>
+      </c>
+      <c r="E15" s="94" t="n">
+        <v>921.1799999999999</v>
+      </c>
+      <c r="F15" s="94" t="n">
+        <v>178.92</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="102" t="inlineStr">
+        <is>
+          <t>En el período quedan 171,18 m³ en el estanque inferior y 178,92 m³ en el superior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="112" t="inlineStr">
+        <is>
+          <t>El 29-09 el superior entrega 13,82 m³ de lo almacenado: Etapa N°5 corre de 18:00 a 23:00 y en varias de esas horas la salida del inferior está en cero. El 01-10 es el día en que más queda en el inferior (36,43 m³). El 24-09 es el día en que más queda en el superior (41,12 m³).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F14"/>
+  <mergeCells count="4">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A17:F17"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;LFundo Zapallar&amp;RAgua almacenada en los estanques</oddHeader>
+    <oddFooter>&amp;LMatriz llena el inferior. La salida del inferior llena el superior.&amp;RPágina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6299,8 +7115,8 @@
   <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A5:F5"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A6:F6"/>
@@ -6322,7 +7138,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F4788"/>
@@ -6899,7 +7715,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00548235"/>
@@ -7266,7 +8082,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
@@ -7642,7 +8458,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C65911"/>
@@ -8186,7 +9002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -8553,223 +9369,4 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00C00000"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="110" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>Hallazgos</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Ordenados para revisar en terreno. El detalle numérico está en las otras hojas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Punto</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Situación</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Qué se encontró</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="53" t="inlineStr">
-        <is>
-          <t>Etapa N°5</t>
-        </is>
-      </c>
-      <c r="C5" s="29" t="inlineStr">
-        <is>
-          <t>Validado</t>
-        </is>
-      </c>
-      <c r="D5" s="74" t="inlineStr">
-        <is>
-          <t>La foto del viernes 02-10 es el mismo Sensus del informe (serie SEN01 2370 9030). La lectura inicial es 5.174 m³ a las 16:54 del 23-09. El viernes a las 08:44 marca 5.369 m³.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="62" customHeight="1">
-      <c r="A6" s="33" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="55" t="inlineStr">
-        <is>
-          <t>Etapa N°5</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>Relojería vs app</t>
-        </is>
-      </c>
-      <c r="D6" s="75" t="inlineStr">
-        <is>
-          <t>Del 23-09 17:00 al 02-10 08:00 (horas de las fotos fuera de la suma) la relojería avanza 195,0 m³ y la app suma 195,6 m³. Error 0,3 % (1 − 195,0/195,6). 207 horas. Desde el 28-09 08:57 (5.225 m³) hasta el viernes la relojería avanza 144 m³ y la app 148,0 m³ (error 2,7 %).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="62" customHeight="1">
-      <c r="A7" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="43" t="inlineStr">
-        <is>
-          <t>Etapa N°5</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>Marzo 2026 no usable</t>
-        </is>
-      </c>
-      <c r="D7" s="57" t="inlineStr">
-        <is>
-          <t>En marzo 2026 Etapa N°5 marca 17.873,4 m³ y la Matriz 1.987,0 m³. Con ese mes, el histórico de WES (32.269,0 m³) supera toda la vida del medidor. Mayo 2026 también queda parejo con la Matriz (Etapa 5 un poco por encima) y conviene mirarlo aparte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="62" customHeight="1">
-      <c r="A8" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="53" t="inlineStr">
-        <is>
-          <t>Matriz ESVAL</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>Medidor identificado</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>La foto de hoy es el mismo Itron Flostar S del informe, en Los Portones 378. El 23-09-2026 a las 17:05 marcaba 384.148,9 m³. Hoy a las 13:22 marca 385.430,8 m³. Relojería 1.281,9 m³ contra app 1.309,6 m³: error 2,1 %, del mismo orden que el 3,7 % del 23–28/09.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="62" customHeight="1">
-      <c r="A9" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="43" t="inlineStr">
-        <is>
-          <t>Matriz ESVAL</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>Telemetría detenida</t>
-        </is>
-      </c>
-      <c r="D9" s="57" t="inlineStr">
-        <is>
-          <t>Última trama 021026 14:14. La foto es de las 13:22, con el punto ya mudo. A las 14:25 llevaba 12 min sin muestras. Etapa N°5, Estanque Inferior y Etapa 1 al 4 tenían trama dentro de los últimos 10 minutos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="62" customHeight="1">
-      <c r="A10" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="55" t="inlineStr">
-        <is>
-          <t>Matriz ESVAL</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="inlineStr">
-        <is>
-          <t>m³ y L/min no cierran</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>No hubo muestras suficientes para recalcular el desfase en esta consulta. Con una sola foto no se sabe cuál de los dos canales está bien.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="62" customHeight="1">
-      <c r="A11" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="49" t="inlineStr">
-        <is>
-          <t>Etapa N°5</t>
-        </is>
-      </c>
-      <c r="C11" s="25" t="inlineStr">
-        <is>
-          <t>Hora de la foto</t>
-        </is>
-      </c>
-      <c r="D11" s="52" t="inlineStr">
-        <is>
-          <t>La validación se pidió con la foto 1 de las 05:00. La hora impresa en esa foto es 08:44. A las 05:00 Etapa N°5 marcaba 0,00 m³, igual que desde la medianoche. A las 08:00 el balde horario es 0,10 m³.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="58" t="inlineStr">
-        <is>
-          <t>Siguiente paso para cerrar la Matriz: segunda lectura del mismo Flostar y revisión en terreno de por qué no volvió a transmitir después de las 13:14.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:D11"/>
-  <mergeCells count="3">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;RPágina &amp;P</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Compare stored volume with the 21 m³ and 30 m³ tank capacities.
The period balance is several times each tank, and 1 October plus 24 and 26 September exceed the useful volume.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
+++ b/reports/Fundo_Zapallar/VALIDACION/Validacion_medidores_Fundo_Zapallar_20261002.xlsx
@@ -44,8 +44,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0&quot; veces&quot;"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -312,7 +313,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -598,10 +599,41 @@
     <xf numFmtId="4" fontId="18" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FECACA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEDD5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -1309,7 +1341,6 @@
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -3834,17 +3865,17 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="111" t="inlineStr">
-        <is>
-          <t>Estanque Inferior. Matriz ESVAL lo llena y el medidor del estanque es su salida. Quedan almacenados 171,18 m³ (1.271,28 − 1.100,10), un 13,5 % de la Matriz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="111" t="inlineStr">
-        <is>
-          <t>Estanque Superior. Lo llena la salida del Inferior. Etapa N°5 y Etapa 1 al 4 son su salida. Quedan almacenados 178,92 m³ (1.100,10 − 921,18), un 16,3 % de la salida del Inferior.</t>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="115" t="inlineStr">
+        <is>
+          <t>Estanque inferior, capacidad 21 m³. En el período el balance suma 171,18 m³ (8,2 veces el estanque). El 01-10 quedan 36,43 m³, un 174 % de la capacidad: ese día no cabe solo como almacenamiento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="115" t="inlineStr">
+        <is>
+          <t>Estanque superior, capacidad 30 m³. En el período el balance suma 178,92 m³ (6,0 veces el estanque). El 24-09 (41,12 m³) y el 26-09 (35,35 m³) superan los 30 m³. El 29-09 entrega 13,82 m³, un 46 % del superior.</t>
         </is>
       </c>
     </row>
@@ -4286,7 +4317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4298,6 +4329,9 @@
     <col width="3" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -4307,14 +4341,14 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="112" t="inlineStr">
         <is>
-          <t>Matriz ESVAL llena el estanque inferior. La salida del inferior llena el estanque superior. Etapa N°5 y Etapa 1 al 4 son la salida del superior. Lo que entra y no sale queda almacenado. Un valor negativo es agua que el estanque entregó de lo que ya tenía.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
+          <t>Matriz ESVAL llena el estanque inferior (21 m³). La salida del inferior llena el estanque superior (30 m³). Etapa N°5 y Etapa 1 al 4 son la salida del superior. El m³ del día solo puede ser cambio de nivel si cabe en el estanque. Si el día supera la capacidad, esa agua no quedó almacenada: rebalsó o salió por un uso que no medimos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="89" t="inlineStr">
         <is>
           <t>Día</t>
@@ -4357,6 +4391,23 @@
           <t>Queda en el superior</t>
         </is>
       </c>
+      <c r="J4" s="89" t="inlineStr">
+        <is>
+          <t>% del inferior
+(21 m³)</t>
+        </is>
+      </c>
+      <c r="K4" s="89" t="inlineStr">
+        <is>
+          <t>% del superior
+(30 m³)</t>
+        </is>
+      </c>
+      <c r="L4" s="89" t="inlineStr">
+        <is>
+          <t>Lectura</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="90" t="inlineStr">
@@ -4385,6 +4436,18 @@
       <c r="I5" s="113" t="n">
         <v>9.35</v>
       </c>
+      <c r="J5" s="116">
+        <f>D5/21</f>
+        <v/>
+      </c>
+      <c r="K5" s="116">
+        <f>F5/30</f>
+        <v/>
+      </c>
+      <c r="L5" s="117">
+        <f>IF(OR(J5&gt;1,K5&gt;1),"Supera la capacidad",IF(K5&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="90" t="inlineStr">
@@ -4413,6 +4476,18 @@
       <c r="I6" s="113" t="n">
         <v>41.12</v>
       </c>
+      <c r="J6" s="116">
+        <f>D6/21</f>
+        <v/>
+      </c>
+      <c r="K6" s="116">
+        <f>F6/30</f>
+        <v/>
+      </c>
+      <c r="L6" s="117">
+        <f>IF(OR(J6&gt;1,K6&gt;1),"Supera la capacidad",IF(K6&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="90" t="inlineStr">
@@ -4441,6 +4516,18 @@
       <c r="I7" s="113" t="n">
         <v>25.28</v>
       </c>
+      <c r="J7" s="116">
+        <f>D7/21</f>
+        <v/>
+      </c>
+      <c r="K7" s="116">
+        <f>F7/30</f>
+        <v/>
+      </c>
+      <c r="L7" s="117">
+        <f>IF(OR(J7&gt;1,K7&gt;1),"Supera la capacidad",IF(K7&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="90" t="inlineStr">
@@ -4469,6 +4556,18 @@
       <c r="I8" s="113" t="n">
         <v>35.35</v>
       </c>
+      <c r="J8" s="116">
+        <f>D8/21</f>
+        <v/>
+      </c>
+      <c r="K8" s="116">
+        <f>F8/30</f>
+        <v/>
+      </c>
+      <c r="L8" s="117">
+        <f>IF(OR(J8&gt;1,K8&gt;1),"Supera la capacidad",IF(K8&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="90" t="inlineStr">
@@ -4497,6 +4596,18 @@
       <c r="I9" s="113" t="n">
         <v>10.75</v>
       </c>
+      <c r="J9" s="116">
+        <f>D9/21</f>
+        <v/>
+      </c>
+      <c r="K9" s="116">
+        <f>F9/30</f>
+        <v/>
+      </c>
+      <c r="L9" s="117">
+        <f>IF(OR(J9&gt;1,K9&gt;1),"Supera la capacidad",IF(K9&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="90" t="inlineStr">
@@ -4525,6 +4636,18 @@
       <c r="I10" s="113" t="n">
         <v>17.99</v>
       </c>
+      <c r="J10" s="116">
+        <f>D10/21</f>
+        <v/>
+      </c>
+      <c r="K10" s="116">
+        <f>F10/30</f>
+        <v/>
+      </c>
+      <c r="L10" s="117">
+        <f>IF(OR(J10&gt;1,K10&gt;1),"Supera la capacidad",IF(K10&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="90" t="inlineStr">
@@ -4553,6 +4676,18 @@
       <c r="I11" s="113" t="n">
         <v>-13.82</v>
       </c>
+      <c r="J11" s="116">
+        <f>D11/21</f>
+        <v/>
+      </c>
+      <c r="K11" s="116">
+        <f>F11/30</f>
+        <v/>
+      </c>
+      <c r="L11" s="117">
+        <f>IF(OR(J11&gt;1,K11&gt;1),"Supera la capacidad",IF(K11&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="90" t="inlineStr">
@@ -4581,6 +4716,18 @@
       <c r="I12" s="113" t="n">
         <v>11.96</v>
       </c>
+      <c r="J12" s="116">
+        <f>D12/21</f>
+        <v/>
+      </c>
+      <c r="K12" s="116">
+        <f>F12/30</f>
+        <v/>
+      </c>
+      <c r="L12" s="117">
+        <f>IF(OR(J12&gt;1,K12&gt;1),"Supera la capacidad",IF(K12&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="90" t="inlineStr">
@@ -4609,6 +4756,18 @@
       <c r="I13" s="113" t="n">
         <v>24.61</v>
       </c>
+      <c r="J13" s="116">
+        <f>D13/21</f>
+        <v/>
+      </c>
+      <c r="K13" s="116">
+        <f>F13/30</f>
+        <v/>
+      </c>
+      <c r="L13" s="117">
+        <f>IF(OR(J13&gt;1,K13&gt;1),"Supera la capacidad",IF(K13&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="90" t="inlineStr">
@@ -4637,6 +4796,18 @@
       <c r="I14" s="113" t="n">
         <v>16.33</v>
       </c>
+      <c r="J14" s="116">
+        <f>D14/21</f>
+        <v/>
+      </c>
+      <c r="K14" s="116">
+        <f>F14/30</f>
+        <v/>
+      </c>
+      <c r="L14" s="117">
+        <f>IF(OR(J14&gt;1,K14&gt;1),"Supera la capacidad",IF(K14&lt;0,"El superior entrega almacenado","Cabe en el estanque"))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="101" t="inlineStr">
@@ -4659,29 +4830,54 @@
       <c r="F15" s="94" t="n">
         <v>178.92</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="102" t="inlineStr">
-        <is>
-          <t>En el período quedan 171,18 m³ en el estanque inferior y 178,92 m³ en el superior.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="48" customHeight="1">
+      <c r="J15" s="118">
+        <f>D15/21</f>
+        <v/>
+      </c>
+      <c r="K15" s="118">
+        <f>F15/30</f>
+        <v/>
+      </c>
+      <c r="L15" s="89" t="inlineStr">
+        <is>
+          <t>Veces la capacidad del período</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="119" t="inlineStr">
+        <is>
+          <t>Capacidad: inferior 21 m³, superior 30 m³. En el período el balance suma 171,18 m³ en el inferior (8,2 veces el estanque) y 178,92 m³ en el superior (6,0 veces el estanque). Esa suma no cabe: el estanque se llena y el resto se va.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
       <c r="A18" s="112" t="inlineStr">
         <is>
-          <t>El 29-09 el superior entrega 13,82 m³ de lo almacenado: Etapa N°5 corre de 18:00 a 23:00 y en varias de esas horas la salida del inferior está en cero. El 01-10 es el día en que más queda en el inferior (36,43 m³). El 24-09 es el día en que más queda en el superior (41,12 m³).</t>
+          <t>Superan la capacidad: el 01-10 en el inferior (36,43 m³, 174 % de 21 m³) y el 24-09 y el 26-09 en el superior (41,12 m³ y 35,35 m³). El 29-09 el superior entrega 13,82 m³, un 46 % de sus 30 m³, y eso sí cabe como bajada de nivel. Varios días del inferior quedan entre 87 % y 97 % del estanque (24, 25, 28 y 30-09): con el estanque ya lleno, el día siguiente no puede seguir guardando ese volumen.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:F14"/>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="A18:L18"/>
   </mergeCells>
+  <conditionalFormatting sqref="J5:K14">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5:K14">
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
@@ -7115,9 +7311,9 @@
   <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A66:F66"/>
-    <mergeCell ref="A5:F5"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A5:F5"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A4:F4"/>

</xml_diff>